<commit_message>
Weekly League Two data update: 2026-09-16
</commit_message>
<xml_diff>
--- a/data/league-two_xg_report.xlsx
+++ b/data/league-two_xg_report.xlsx
@@ -2633,22 +2633,22 @@
         <v>1.41</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>1.33</v>
+        <v>1.44</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>1.69</v>
+        <v>1.9</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>-0.2</v>
+        <v>-0.09</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>0.28</v>
+        <v>0.49</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>0.34</v>
+        <v>0.36</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>-0.04</v>
+        <v>-0.01</v>
       </c>
       <c r="N7" s="4">
         <f>(H7-I7)-(F7-G7)</f>
@@ -4707,7 +4707,7 @@
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
-    <col width="6" customWidth="1" min="13" max="13"/>
+    <col width="5" customWidth="1" min="13" max="13"/>
     <col width="6" customWidth="1" min="14" max="14"/>
     <col width="6" customWidth="1" min="15" max="15"/>
   </cols>
@@ -5093,22 +5093,22 @@
         <v>1.26</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>1.28</v>
+        <v>1.49</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.9</v>
+        <v>1.25</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0</v>
+        <v>0.21</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>-0.36</v>
+        <v>-0.01</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>-0.03</v>
+        <v>0.03</v>
       </c>
       <c r="N7" s="4">
         <f>(H7-I7)-(F7-G7)</f>
@@ -5708,22 +5708,22 @@
         <v>1.34</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>1.23</v>
+        <v>1.44</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.09</v>
+        <v>0.11</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>-0.29</v>
+        <v>-0.08</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>-1.25</v>
+        <v>-1.23</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>0.14</v>
+        <v>0.17</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="N7" s="4">
         <f>(H7-I7)-(F7-G7)</f>
@@ -12197,22 +12197,22 @@
         <v>2.02</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.58</v>
+        <v>0.49</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>2.42</v>
+        <v>2.59</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>-0.49</v>
+        <v>-0.58</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>0.4</v>
+        <v>0.57</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>-0.2</v>
+        <v>-0.22</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="N7" s="4">
         <f>(H7-I7)-(F7-G7)</f>
@@ -12812,22 +12812,22 @@
         <v>1.28</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.9</v>
+        <v>1.25</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>1.28</v>
+        <v>1.49</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>-0.36</v>
+        <v>-0.01</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>0</v>
+        <v>0.21</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>-0.15</v>
+        <v>-0.09</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0.26</v>
+        <v>0.29</v>
       </c>
       <c r="N7" s="4">
         <f>(H7-I7)-(F7-G7)</f>
@@ -14042,22 +14042,22 @@
         <v>1.07</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>2.42</v>
+        <v>2.59</v>
       </c>
       <c r="I7" s="4" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>-0.58</v>
+      </c>
+      <c r="L7" s="4" t="n">
         <v>0.58</v>
       </c>
-      <c r="J7" s="4" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>-0.49</v>
-      </c>
-      <c r="L7" s="4" t="n">
-        <v>0.55</v>
-      </c>
       <c r="M7" s="4" t="n">
-        <v>-0.01</v>
+        <v>-0.03</v>
       </c>
       <c r="N7" s="4">
         <f>(H7-I7)-(F7-G7)</f>
@@ -16368,70 +16368,70 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Cheltenham Town</t>
+          <t>Oldham Athletic</t>
         </is>
       </c>
       <c r="B12" s="5">
-        <f>'Cheltenham Town'!$E$15</f>
+        <f>'Oldham Athletic'!$E$15</f>
         <v/>
       </c>
       <c r="C12" s="4">
-        <f>'Cheltenham Town'!$N$2</f>
+        <f>'Oldham Athletic'!$N$2</f>
         <v/>
       </c>
       <c r="D12" s="4">
-        <f>'Cheltenham Town'!$N$3</f>
+        <f>'Oldham Athletic'!$N$3</f>
         <v/>
       </c>
       <c r="E12" s="4">
-        <f>'Cheltenham Town'!$N$4</f>
+        <f>'Oldham Athletic'!$N$4</f>
         <v/>
       </c>
       <c r="F12" s="4">
-        <f>'Cheltenham Town'!$N$5</f>
+        <f>'Oldham Athletic'!$N$5</f>
         <v/>
       </c>
       <c r="G12" s="4">
-        <f>'Cheltenham Town'!$N$6</f>
+        <f>'Oldham Athletic'!$N$6</f>
         <v/>
       </c>
       <c r="H12" s="4">
-        <f>'Cheltenham Town'!$N$7</f>
+        <f>'Oldham Athletic'!$N$7</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Oldham Athletic</t>
+          <t>Cheltenham Town</t>
         </is>
       </c>
       <c r="B13" s="5">
-        <f>'Oldham Athletic'!$E$15</f>
+        <f>'Cheltenham Town'!$E$15</f>
         <v/>
       </c>
       <c r="C13" s="4">
-        <f>'Oldham Athletic'!$N$2</f>
+        <f>'Cheltenham Town'!$N$2</f>
         <v/>
       </c>
       <c r="D13" s="4">
-        <f>'Oldham Athletic'!$N$3</f>
+        <f>'Cheltenham Town'!$N$3</f>
         <v/>
       </c>
       <c r="E13" s="4">
-        <f>'Oldham Athletic'!$N$4</f>
+        <f>'Cheltenham Town'!$N$4</f>
         <v/>
       </c>
       <c r="F13" s="4">
-        <f>'Oldham Athletic'!$N$5</f>
+        <f>'Cheltenham Town'!$N$5</f>
         <v/>
       </c>
       <c r="G13" s="4">
-        <f>'Oldham Athletic'!$N$6</f>
+        <f>'Cheltenham Town'!$N$6</f>
         <v/>
       </c>
       <c r="H13" s="4">
-        <f>'Oldham Athletic'!$N$7</f>
+        <f>'Cheltenham Town'!$N$7</f>
         <v/>
       </c>
     </row>
@@ -16718,70 +16718,70 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>York</t>
+          <t>Bristol Rvs</t>
         </is>
       </c>
       <c r="B22" s="5">
-        <f>'York'!$E$15</f>
+        <f>'Bristol Rvs'!$E$15</f>
         <v/>
       </c>
       <c r="C22" s="4">
-        <f>'York'!$N$2</f>
+        <f>'Bristol Rvs'!$N$2</f>
         <v/>
       </c>
       <c r="D22" s="4">
-        <f>'York'!$N$3</f>
+        <f>'Bristol Rvs'!$N$3</f>
         <v/>
       </c>
       <c r="E22" s="4">
-        <f>'York'!$N$4</f>
+        <f>'Bristol Rvs'!$N$4</f>
         <v/>
       </c>
       <c r="F22" s="4">
-        <f>'York'!$N$5</f>
+        <f>'Bristol Rvs'!$N$5</f>
         <v/>
       </c>
       <c r="G22" s="4">
-        <f>'York'!$N$6</f>
+        <f>'Bristol Rvs'!$N$6</f>
         <v/>
       </c>
       <c r="H22" s="4">
-        <f>'York'!$N$7</f>
+        <f>'Bristol Rvs'!$N$7</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Bristol Rvs</t>
+          <t>York</t>
         </is>
       </c>
       <c r="B23" s="5">
-        <f>'Bristol Rvs'!$E$15</f>
+        <f>'York'!$E$15</f>
         <v/>
       </c>
       <c r="C23" s="4">
-        <f>'Bristol Rvs'!$N$2</f>
+        <f>'York'!$N$2</f>
         <v/>
       </c>
       <c r="D23" s="4">
-        <f>'Bristol Rvs'!$N$3</f>
+        <f>'York'!$N$3</f>
         <v/>
       </c>
       <c r="E23" s="4">
-        <f>'Bristol Rvs'!$N$4</f>
+        <f>'York'!$N$4</f>
         <v/>
       </c>
       <c r="F23" s="4">
-        <f>'Bristol Rvs'!$N$5</f>
+        <f>'York'!$N$5</f>
         <v/>
       </c>
       <c r="G23" s="4">
-        <f>'Bristol Rvs'!$N$6</f>
+        <f>'York'!$N$6</f>
         <v/>
       </c>
       <c r="H23" s="4">
-        <f>'Bristol Rvs'!$N$7</f>
+        <f>'York'!$N$7</f>
         <v/>
       </c>
     </row>
@@ -17182,70 +17182,70 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Swindon Town</t>
+          <t>Crewe Alexandra</t>
         </is>
       </c>
       <c r="B9" s="5">
-        <f>'Swindon Town'!$E$16</f>
+        <f>'Crewe Alexandra'!$E$16</f>
         <v/>
       </c>
       <c r="C9" s="4">
-        <f>'Swindon Town'!$O$2</f>
+        <f>'Crewe Alexandra'!$O$2</f>
         <v/>
       </c>
       <c r="D9" s="4">
-        <f>'Swindon Town'!$O$3</f>
+        <f>'Crewe Alexandra'!$O$3</f>
         <v/>
       </c>
       <c r="E9" s="4">
-        <f>'Swindon Town'!$O$4</f>
+        <f>'Crewe Alexandra'!$O$4</f>
         <v/>
       </c>
       <c r="F9" s="4">
-        <f>'Swindon Town'!$O$5</f>
+        <f>'Crewe Alexandra'!$O$5</f>
         <v/>
       </c>
       <c r="G9" s="4">
-        <f>'Swindon Town'!$O$6</f>
+        <f>'Crewe Alexandra'!$O$6</f>
         <v/>
       </c>
       <c r="H9" s="4">
-        <f>'Swindon Town'!$O$7</f>
+        <f>'Crewe Alexandra'!$O$7</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Crewe Alexandra</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="B10" s="5">
-        <f>'Crewe Alexandra'!$E$16</f>
+        <f>'Swindon Town'!$E$16</f>
         <v/>
       </c>
       <c r="C10" s="4">
-        <f>'Crewe Alexandra'!$O$2</f>
+        <f>'Swindon Town'!$O$2</f>
         <v/>
       </c>
       <c r="D10" s="4">
-        <f>'Crewe Alexandra'!$O$3</f>
+        <f>'Swindon Town'!$O$3</f>
         <v/>
       </c>
       <c r="E10" s="4">
-        <f>'Crewe Alexandra'!$O$4</f>
+        <f>'Swindon Town'!$O$4</f>
         <v/>
       </c>
       <c r="F10" s="4">
-        <f>'Crewe Alexandra'!$O$5</f>
+        <f>'Swindon Town'!$O$5</f>
         <v/>
       </c>
       <c r="G10" s="4">
-        <f>'Crewe Alexandra'!$O$6</f>
+        <f>'Swindon Town'!$O$6</f>
         <v/>
       </c>
       <c r="H10" s="4">
-        <f>'Crewe Alexandra'!$O$7</f>
+        <f>'Swindon Town'!$O$7</f>
         <v/>
       </c>
     </row>
@@ -17287,140 +17287,140 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Tranmere Rovers</t>
+          <t>Oldham Athletic</t>
         </is>
       </c>
       <c r="B12" s="5">
-        <f>'Tranmere Rovers'!$E$16</f>
+        <f>'Oldham Athletic'!$E$16</f>
         <v/>
       </c>
       <c r="C12" s="4">
-        <f>'Tranmere Rovers'!$O$2</f>
+        <f>'Oldham Athletic'!$O$2</f>
         <v/>
       </c>
       <c r="D12" s="4">
-        <f>'Tranmere Rovers'!$O$3</f>
+        <f>'Oldham Athletic'!$O$3</f>
         <v/>
       </c>
       <c r="E12" s="4">
-        <f>'Tranmere Rovers'!$O$4</f>
+        <f>'Oldham Athletic'!$O$4</f>
         <v/>
       </c>
       <c r="F12" s="4">
-        <f>'Tranmere Rovers'!$O$5</f>
+        <f>'Oldham Athletic'!$O$5</f>
         <v/>
       </c>
       <c r="G12" s="4">
-        <f>'Tranmere Rovers'!$O$6</f>
+        <f>'Oldham Athletic'!$O$6</f>
         <v/>
       </c>
       <c r="H12" s="4">
-        <f>'Tranmere Rovers'!$O$7</f>
+        <f>'Oldham Athletic'!$O$7</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Bristol Rvs</t>
+          <t>Colchester United</t>
         </is>
       </c>
       <c r="B13" s="5">
-        <f>'Bristol Rvs'!$E$16</f>
+        <f>'Colchester United'!$E$16</f>
         <v/>
       </c>
       <c r="C13" s="4">
-        <f>'Bristol Rvs'!$O$2</f>
+        <f>'Colchester United'!$O$2</f>
         <v/>
       </c>
       <c r="D13" s="4">
-        <f>'Bristol Rvs'!$O$3</f>
+        <f>'Colchester United'!$O$3</f>
         <v/>
       </c>
       <c r="E13" s="4">
-        <f>'Bristol Rvs'!$O$4</f>
+        <f>'Colchester United'!$O$4</f>
         <v/>
       </c>
       <c r="F13" s="4">
-        <f>'Bristol Rvs'!$O$5</f>
+        <f>'Colchester United'!$O$5</f>
         <v/>
       </c>
       <c r="G13" s="4">
-        <f>'Bristol Rvs'!$O$6</f>
+        <f>'Colchester United'!$O$6</f>
         <v/>
       </c>
       <c r="H13" s="4">
-        <f>'Bristol Rvs'!$O$7</f>
+        <f>'Colchester United'!$O$7</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Oldham Athletic</t>
+          <t>Tranmere Rovers</t>
         </is>
       </c>
       <c r="B14" s="5">
-        <f>'Oldham Athletic'!$E$16</f>
+        <f>'Tranmere Rovers'!$E$16</f>
         <v/>
       </c>
       <c r="C14" s="4">
-        <f>'Oldham Athletic'!$O$2</f>
+        <f>'Tranmere Rovers'!$O$2</f>
         <v/>
       </c>
       <c r="D14" s="4">
-        <f>'Oldham Athletic'!$O$3</f>
+        <f>'Tranmere Rovers'!$O$3</f>
         <v/>
       </c>
       <c r="E14" s="4">
-        <f>'Oldham Athletic'!$O$4</f>
+        <f>'Tranmere Rovers'!$O$4</f>
         <v/>
       </c>
       <c r="F14" s="4">
-        <f>'Oldham Athletic'!$O$5</f>
+        <f>'Tranmere Rovers'!$O$5</f>
         <v/>
       </c>
       <c r="G14" s="4">
-        <f>'Oldham Athletic'!$O$6</f>
+        <f>'Tranmere Rovers'!$O$6</f>
         <v/>
       </c>
       <c r="H14" s="4">
-        <f>'Oldham Athletic'!$O$7</f>
+        <f>'Tranmere Rovers'!$O$7</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Colchester United</t>
+          <t>Bristol Rvs</t>
         </is>
       </c>
       <c r="B15" s="5">
-        <f>'Colchester United'!$E$16</f>
+        <f>'Bristol Rvs'!$E$16</f>
         <v/>
       </c>
       <c r="C15" s="4">
-        <f>'Colchester United'!$O$2</f>
+        <f>'Bristol Rvs'!$O$2</f>
         <v/>
       </c>
       <c r="D15" s="4">
-        <f>'Colchester United'!$O$3</f>
+        <f>'Bristol Rvs'!$O$3</f>
         <v/>
       </c>
       <c r="E15" s="4">
-        <f>'Colchester United'!$O$4</f>
+        <f>'Bristol Rvs'!$O$4</f>
         <v/>
       </c>
       <c r="F15" s="4">
-        <f>'Colchester United'!$O$5</f>
+        <f>'Bristol Rvs'!$O$5</f>
         <v/>
       </c>
       <c r="G15" s="4">
-        <f>'Colchester United'!$O$6</f>
+        <f>'Bristol Rvs'!$O$6</f>
         <v/>
       </c>
       <c r="H15" s="4">
-        <f>'Colchester United'!$O$7</f>
+        <f>'Bristol Rvs'!$O$7</f>
         <v/>
       </c>
     </row>
@@ -17462,175 +17462,175 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Fleetwood Town</t>
         </is>
       </c>
       <c r="B17" s="5">
-        <f>'Crawley Town'!$E$16</f>
+        <f>'Fleetwood Town'!$E$16</f>
         <v/>
       </c>
       <c r="C17" s="4">
-        <f>'Crawley Town'!$O$2</f>
+        <f>'Fleetwood Town'!$O$2</f>
         <v/>
       </c>
       <c r="D17" s="4">
-        <f>'Crawley Town'!$O$3</f>
+        <f>'Fleetwood Town'!$O$3</f>
         <v/>
       </c>
       <c r="E17" s="4">
-        <f>'Crawley Town'!$O$4</f>
+        <f>'Fleetwood Town'!$O$4</f>
         <v/>
       </c>
       <c r="F17" s="4">
-        <f>'Crawley Town'!$O$5</f>
+        <f>'Fleetwood Town'!$O$5</f>
         <v/>
       </c>
       <c r="G17" s="4">
-        <f>'Crawley Town'!$O$6</f>
+        <f>'Fleetwood Town'!$O$6</f>
         <v/>
       </c>
       <c r="H17" s="4">
-        <f>'Crawley Town'!$O$7</f>
+        <f>'Fleetwood Town'!$O$7</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Cheltenham Town</t>
+          <t>Rotherham United</t>
         </is>
       </c>
       <c r="B18" s="5">
-        <f>'Cheltenham Town'!$E$16</f>
+        <f>'Rotherham United'!$E$16</f>
         <v/>
       </c>
       <c r="C18" s="4">
-        <f>'Cheltenham Town'!$O$2</f>
+        <f>'Rotherham United'!$O$2</f>
         <v/>
       </c>
       <c r="D18" s="4">
-        <f>'Cheltenham Town'!$O$3</f>
+        <f>'Rotherham United'!$O$3</f>
         <v/>
       </c>
       <c r="E18" s="4">
-        <f>'Cheltenham Town'!$O$4</f>
+        <f>'Rotherham United'!$O$4</f>
         <v/>
       </c>
       <c r="F18" s="4">
-        <f>'Cheltenham Town'!$O$5</f>
+        <f>'Rotherham United'!$O$5</f>
         <v/>
       </c>
       <c r="G18" s="4">
-        <f>'Cheltenham Town'!$O$6</f>
+        <f>'Rotherham United'!$O$6</f>
         <v/>
       </c>
       <c r="H18" s="4">
-        <f>'Cheltenham Town'!$O$7</f>
+        <f>'Rotherham United'!$O$7</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Fleetwood Town</t>
+          <t>Barnet</t>
         </is>
       </c>
       <c r="B19" s="5">
-        <f>'Fleetwood Town'!$E$16</f>
+        <f>'Barnet'!$E$16</f>
         <v/>
       </c>
       <c r="C19" s="4">
-        <f>'Fleetwood Town'!$O$2</f>
+        <f>'Barnet'!$O$2</f>
         <v/>
       </c>
       <c r="D19" s="4">
-        <f>'Fleetwood Town'!$O$3</f>
+        <f>'Barnet'!$O$3</f>
         <v/>
       </c>
       <c r="E19" s="4">
-        <f>'Fleetwood Town'!$O$4</f>
+        <f>'Barnet'!$O$4</f>
         <v/>
       </c>
       <c r="F19" s="4">
-        <f>'Fleetwood Town'!$O$5</f>
+        <f>'Barnet'!$O$5</f>
         <v/>
       </c>
       <c r="G19" s="4">
-        <f>'Fleetwood Town'!$O$6</f>
+        <f>'Barnet'!$O$6</f>
         <v/>
       </c>
       <c r="H19" s="4">
-        <f>'Fleetwood Town'!$O$7</f>
+        <f>'Barnet'!$O$7</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Rotherham United</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="B20" s="5">
-        <f>'Rotherham United'!$E$16</f>
+        <f>'Crawley Town'!$E$16</f>
         <v/>
       </c>
       <c r="C20" s="4">
-        <f>'Rotherham United'!$O$2</f>
+        <f>'Crawley Town'!$O$2</f>
         <v/>
       </c>
       <c r="D20" s="4">
-        <f>'Rotherham United'!$O$3</f>
+        <f>'Crawley Town'!$O$3</f>
         <v/>
       </c>
       <c r="E20" s="4">
-        <f>'Rotherham United'!$O$4</f>
+        <f>'Crawley Town'!$O$4</f>
         <v/>
       </c>
       <c r="F20" s="4">
-        <f>'Rotherham United'!$O$5</f>
+        <f>'Crawley Town'!$O$5</f>
         <v/>
       </c>
       <c r="G20" s="4">
-        <f>'Rotherham United'!$O$6</f>
+        <f>'Crawley Town'!$O$6</f>
         <v/>
       </c>
       <c r="H20" s="4">
-        <f>'Rotherham United'!$O$7</f>
+        <f>'Crawley Town'!$O$7</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Barnet</t>
+          <t>Cheltenham Town</t>
         </is>
       </c>
       <c r="B21" s="5">
-        <f>'Barnet'!$E$16</f>
+        <f>'Cheltenham Town'!$E$16</f>
         <v/>
       </c>
       <c r="C21" s="4">
-        <f>'Barnet'!$O$2</f>
+        <f>'Cheltenham Town'!$O$2</f>
         <v/>
       </c>
       <c r="D21" s="4">
-        <f>'Barnet'!$O$3</f>
+        <f>'Cheltenham Town'!$O$3</f>
         <v/>
       </c>
       <c r="E21" s="4">
-        <f>'Barnet'!$O$4</f>
+        <f>'Cheltenham Town'!$O$4</f>
         <v/>
       </c>
       <c r="F21" s="4">
-        <f>'Barnet'!$O$5</f>
+        <f>'Cheltenham Town'!$O$5</f>
         <v/>
       </c>
       <c r="G21" s="4">
-        <f>'Barnet'!$O$6</f>
+        <f>'Cheltenham Town'!$O$6</f>
         <v/>
       </c>
       <c r="H21" s="4">
-        <f>'Barnet'!$O$7</f>
+        <f>'Cheltenham Town'!$O$7</f>
         <v/>
       </c>
     </row>
@@ -19417,22 +19417,22 @@
         <v>1.52</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.09</v>
+        <v>0.11</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>1.23</v>
+        <v>1.44</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>-1.25</v>
+        <v>-1.23</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>-0.29</v>
+        <v>-0.08</v>
       </c>
       <c r="L7" s="4" t="n">
         <v>0.38</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>-0.2</v>
+        <v>-0.16</v>
       </c>
       <c r="N7" s="4">
         <f>(H7-I7)-(F7-G7)</f>
@@ -20032,22 +20032,22 @@
         <v>1.53</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>1.69</v>
+        <v>1.9</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>1.33</v>
+        <v>1.44</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0.28</v>
+        <v>0.49</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>-0.2</v>
+        <v>-0.09</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>0.15</v>
+        <v>0.18</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0.17</v>
+        <v>0.19</v>
       </c>
       <c r="N7" s="4">
         <f>(H7-I7)-(F7-G7)</f>

</xml_diff>

<commit_message>
Weekly League Two data update: 2026-09-24
</commit_message>
<xml_diff>
--- a/data/league-two_xg_report.xlsx
+++ b/data/league-two_xg_report.xlsx
@@ -1459,45 +1459,45 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Colchester United</t>
+          <t>Barnet</t>
         </is>
       </c>
       <c r="B14" s="14" t="n">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="C14" s="9" t="n">
-        <v>2.02</v>
+        <v>0.46</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>0.1</v>
+        <v>-0.57</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>0.28</v>
+        <v>0.74</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>-1.66</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Barnet</t>
+          <t>Colchester United</t>
         </is>
       </c>
       <c r="B15" s="14" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>0.46</v>
+        <v>2.02</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>-0.57</v>
+        <v>0.1</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>0.74</v>
+        <v>0.28</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>-0.03</v>
+        <v>-1.66</v>
       </c>
     </row>
     <row r="16">
@@ -1609,7 +1609,7 @@
         </is>
       </c>
       <c r="B21" s="14" t="n">
-        <v>-0.77</v>
+        <v>-0.84</v>
       </c>
       <c r="C21" s="9" t="n">
         <v>-2.23</v>
@@ -1621,7 +1621,7 @@
         <v>-0.98</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>-0.58</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="22">
@@ -2224,7 +2224,7 @@
         </is>
       </c>
       <c r="B23" s="14" t="n">
-        <v>-0.73</v>
+        <v>-0.65</v>
       </c>
       <c r="C23" s="9" t="n">
         <v>-0.19</v>
@@ -2236,7 +2236,7 @@
         <v>-1.15</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>0.58</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="24">
@@ -2246,7 +2246,7 @@
         </is>
       </c>
       <c r="B24" s="14" t="n">
-        <v>-0.75</v>
+        <v>-0.8</v>
       </c>
       <c r="C24" s="9" t="n">
         <v>-0.38</v>
@@ -2258,7 +2258,7 @@
         <v>-1.97</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>0.03</v>
+        <v>-0.16</v>
       </c>
     </row>
     <row r="25">
@@ -2590,86 +2590,86 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>York</t>
+          <t>Fleetwood Town</t>
         </is>
       </c>
       <c r="B7" s="14">
-        <f>'York'!$E$24</f>
+        <f>'Fleetwood Town'!$E$24</f>
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>'York'!$S$2</f>
+        <f>'Fleetwood Town'!$S$2</f>
         <v/>
       </c>
       <c r="D7" s="9">
-        <f>'York'!$S$3</f>
+        <f>'Fleetwood Town'!$S$3</f>
         <v/>
       </c>
       <c r="E7" s="9">
-        <f>'York'!$S$4</f>
+        <f>'Fleetwood Town'!$S$4</f>
         <v/>
       </c>
       <c r="F7" s="9">
-        <f>'York'!$S$5</f>
+        <f>'Fleetwood Town'!$S$5</f>
         <v/>
       </c>
       <c r="G7" s="9">
-        <f>'York'!$S$6</f>
+        <f>'Fleetwood Town'!$S$6</f>
         <v/>
       </c>
       <c r="H7" s="9">
-        <f>'York'!$S$7</f>
+        <f>'Fleetwood Town'!$S$7</f>
         <v/>
       </c>
       <c r="I7" s="9">
-        <f>'York'!$S$8</f>
+        <f>'Fleetwood Town'!$S$8</f>
         <v/>
       </c>
       <c r="J7" s="14">
-        <f>'York'!$E$25</f>
+        <f>'Fleetwood Town'!$E$25</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Fleetwood Town</t>
+          <t>York</t>
         </is>
       </c>
       <c r="B8" s="14">
-        <f>'Fleetwood Town'!$E$24</f>
+        <f>'York'!$E$24</f>
         <v/>
       </c>
       <c r="C8" s="9">
-        <f>'Fleetwood Town'!$S$2</f>
+        <f>'York'!$S$2</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>'Fleetwood Town'!$S$3</f>
+        <f>'York'!$S$3</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>'Fleetwood Town'!$S$4</f>
+        <f>'York'!$S$4</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>'Fleetwood Town'!$S$5</f>
+        <f>'York'!$S$5</f>
         <v/>
       </c>
       <c r="G8" s="9">
-        <f>'Fleetwood Town'!$S$6</f>
+        <f>'York'!$S$6</f>
         <v/>
       </c>
       <c r="H8" s="9">
-        <f>'Fleetwood Town'!$S$7</f>
+        <f>'York'!$S$7</f>
         <v/>
       </c>
       <c r="I8" s="9">
-        <f>'Fleetwood Town'!$S$8</f>
+        <f>'York'!$S$8</f>
         <v/>
       </c>
       <c r="J8" s="14">
-        <f>'Fleetwood Town'!$E$25</f>
+        <f>'York'!$E$25</f>
         <v/>
       </c>
     </row>
@@ -4272,78 +4272,78 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Fleetwood Town</t>
+          <t>Northampton Town</t>
         </is>
       </c>
       <c r="B22" s="14">
-        <f>'Fleetwood Town'!$E$32</f>
+        <f>'Northampton Town'!$E$32</f>
         <v/>
       </c>
       <c r="C22" s="9">
-        <f>'Fleetwood Town'!$V$2</f>
+        <f>'Northampton Town'!$V$2</f>
         <v/>
       </c>
       <c r="D22" s="9">
-        <f>'Fleetwood Town'!$V$3</f>
+        <f>'Northampton Town'!$V$3</f>
         <v/>
       </c>
       <c r="E22" s="9">
-        <f>'Fleetwood Town'!$V$4</f>
+        <f>'Northampton Town'!$V$4</f>
         <v/>
       </c>
       <c r="F22" s="9">
-        <f>'Fleetwood Town'!$V$5</f>
+        <f>'Northampton Town'!$V$5</f>
         <v/>
       </c>
       <c r="G22" s="9">
-        <f>'Fleetwood Town'!$V$6</f>
+        <f>'Northampton Town'!$V$6</f>
         <v/>
       </c>
       <c r="H22" s="9">
-        <f>'Fleetwood Town'!$V$7</f>
+        <f>'Northampton Town'!$V$7</f>
         <v/>
       </c>
       <c r="I22" s="9">
-        <f>'Fleetwood Town'!$V$8</f>
+        <f>'Northampton Town'!$V$8</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Northampton Town</t>
+          <t>Fleetwood Town</t>
         </is>
       </c>
       <c r="B23" s="14">
-        <f>'Northampton Town'!$E$32</f>
+        <f>'Fleetwood Town'!$E$32</f>
         <v/>
       </c>
       <c r="C23" s="9">
-        <f>'Northampton Town'!$V$2</f>
+        <f>'Fleetwood Town'!$V$2</f>
         <v/>
       </c>
       <c r="D23" s="9">
-        <f>'Northampton Town'!$V$3</f>
+        <f>'Fleetwood Town'!$V$3</f>
         <v/>
       </c>
       <c r="E23" s="9">
-        <f>'Northampton Town'!$V$4</f>
+        <f>'Fleetwood Town'!$V$4</f>
         <v/>
       </c>
       <c r="F23" s="9">
-        <f>'Northampton Town'!$V$5</f>
+        <f>'Fleetwood Town'!$V$5</f>
         <v/>
       </c>
       <c r="G23" s="9">
-        <f>'Northampton Town'!$V$6</f>
+        <f>'Fleetwood Town'!$V$6</f>
         <v/>
       </c>
       <c r="H23" s="9">
-        <f>'Northampton Town'!$V$7</f>
+        <f>'Fleetwood Town'!$V$7</f>
         <v/>
       </c>
       <c r="I23" s="9">
-        <f>'Northampton Town'!$V$8</f>
+        <f>'Fleetwood Town'!$V$8</f>
         <v/>
       </c>
     </row>
@@ -4590,25 +4590,25 @@
         <v>0.8100000000000001</v>
       </c>
       <c r="E3" s="10" t="n">
-        <v>-0.14</v>
+        <v>-0.11</v>
       </c>
       <c r="F3" s="10" t="n">
-        <v>-0.67</v>
+        <v>-0.7</v>
       </c>
       <c r="G3" s="10" t="n">
-        <v>1.34</v>
+        <v>1.4</v>
       </c>
       <c r="H3" s="10" t="n">
         <v>2.95</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>0.41</v>
+        <v>0.52</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>0.33</v>
+        <v>0.44</v>
       </c>
       <c r="K3" s="10" t="n">
-        <v>3.69</v>
+        <v>3.91</v>
       </c>
       <c r="L3" s="8" t="inlineStr"/>
     </row>
@@ -4704,37 +4704,37 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Salford City</t>
+          <t>Accrington Stanley</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Swindon Town</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="D6" s="9" t="n">
-        <v>1.03</v>
+        <v>0.43</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>-0.7</v>
+        <v>0.2</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>-0.19</v>
+        <v>0.15</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>0.52</v>
+        <v>0.48</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>3.14</v>
+        <v>2.71</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>-0.28</v>
+        <v>0.67</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>-0.14</v>
+        <v>-0.36</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>2.72</v>
+        <v>3.02</v>
       </c>
       <c r="L6" s="6" t="inlineStr"/>
     </row>
@@ -4746,37 +4746,37 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Accrington Stanley</t>
+          <t>Salford City</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="D7" s="10" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="G7" s="10" t="n">
         <v>0.43</v>
       </c>
-      <c r="E7" s="10" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F7" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="G7" s="10" t="n">
-        <v>0.48</v>
-      </c>
       <c r="H7" s="10" t="n">
-        <v>2.71</v>
+        <v>3.14</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>0.67</v>
+        <v>-0.35</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>-0.36</v>
+        <v>-0.21</v>
       </c>
       <c r="K7" s="10" t="n">
-        <v>3.02</v>
+        <v>2.58</v>
       </c>
       <c r="L7" s="8" t="inlineStr"/>
     </row>
@@ -5679,16 +5679,16 @@
         <v>0.37</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>-0.73</v>
+        <v>-0.78</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>0.3</v>
+        <v>0.22</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.26</v>
+        <v>0.24</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -5767,10 +5767,10 @@
         <v>-0.52</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>0.23</v>
+        <v>0.21</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -6543,16 +6543,16 @@
         <v>-0.26</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>0.28</v>
+        <v>0.34</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>0.28</v>
+        <v>0.34</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -6634,7 +6634,7 @@
         <v>0.03</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>0.46</v>
+        <v>0.49</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -6716,7 +6716,7 @@
         <v>0.12</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.53</v>
+        <v>0.55</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -6798,7 +6798,7 @@
         <v>-0.01</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.4</v>
+        <v>0.41</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -6880,7 +6880,7 @@
         <v>0.25</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.37</v>
+        <v>0.38</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -6962,7 +6962,7 @@
         <v>0.24</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -7017,34 +7017,34 @@
         <v>1.07</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>2.06</v>
+        <v>2.55</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>1.28</v>
+        <v>1.58</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0.18</v>
+        <v>0.67</v>
       </c>
       <c r="K8" s="9" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="L8" s="9" t="n">
         <v>0.21</v>
       </c>
-      <c r="L8" s="9" t="n">
-        <v>0.12</v>
-      </c>
       <c r="M8" s="9" t="n">
-        <v>0.36</v>
+        <v>0.41</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-0.38</v>
+        <v>0.11</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>0.45</v>
+        <v>0.75</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.18</v>
+        <v>0.26</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>0.18</v>
+        <v>0.23</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -7055,16 +7055,16 @@
         <v/>
       </c>
       <c r="T8" s="9" t="n">
-        <v>1.87</v>
+        <v>1.95</v>
       </c>
       <c r="U8" s="9" t="n">
         <v>1.91</v>
       </c>
       <c r="V8" s="9" t="n">
-        <v>-0.04</v>
+        <v>0.03</v>
       </c>
       <c r="W8" s="9" t="n">
-        <v>11.41</v>
+        <v>11.48</v>
       </c>
       <c r="X8" s="9" t="n">
         <v>12.15</v>
@@ -7384,16 +7384,16 @@
         <v>5</v>
       </c>
       <c r="E36" s="19" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="F36" s="19" t="n">
-        <v>0.22</v>
+        <v>0.31</v>
       </c>
       <c r="G36" s="19" t="n">
-        <v>0.38</v>
+        <v>0.58</v>
       </c>
       <c r="H36" s="19" t="n">
-        <v>0.21</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="37">
@@ -7440,13 +7440,13 @@
         <v>10</v>
       </c>
       <c r="E38" s="21" t="n">
-        <v>-0.14</v>
+        <v>-0.11</v>
       </c>
       <c r="F38" s="21" t="n">
-        <v>-0.03</v>
+        <v>0.16</v>
       </c>
       <c r="G38" s="21" t="n">
-        <v>0.41</v>
+        <v>0.52</v>
       </c>
       <c r="H38" s="21" t="n">
         <v>0.22</v>
@@ -9173,13 +9173,13 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>-0.62</v>
+        <v>-0.61</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>-0.22</v>
+        <v>-0.19</v>
       </c>
       <c r="Q3" s="10" t="n">
         <v>-0.14</v>
@@ -9255,16 +9255,16 @@
         <v>0.14</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>0.68</v>
+        <v>0.63</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>0.18</v>
+        <v>0.1</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.03</v>
+        <v>-0.06</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -9346,7 +9346,7 @@
         <v>0.12</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -9428,7 +9428,7 @@
         <v>0.1</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>-0.03</v>
+        <v>-0.04</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -9507,10 +9507,10 @@
         <v>-0.44</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>-0.1</v>
+        <v>-0.11</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -9589,10 +9589,10 @@
         <v>-0.8100000000000001</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.29</v>
+        <v>-0.3</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -10365,16 +10365,16 @@
         <v>0.16</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>0.04</v>
+        <v>-0.04</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>0.38</v>
+        <v>0.33</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>0.04</v>
+        <v>-0.04</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>0.38</v>
+        <v>0.33</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -10447,13 +10447,13 @@
         <v>-0.41</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>1.21</v>
+        <v>1.22</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>-0.57</v>
+        <v>-0.51</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>0.63</v>
+        <v>0.59</v>
       </c>
       <c r="Q3" s="10" t="n">
         <v>-0.09</v>
@@ -10535,10 +10535,10 @@
         <v>1.4</v>
       </c>
       <c r="P4" s="9" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="Q4" s="9" t="n">
         <v>0.41</v>
-      </c>
-      <c r="Q4" s="9" t="n">
-        <v>0.4</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -10617,7 +10617,7 @@
         <v>-0.63</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>0.42</v>
+        <v>0.4</v>
       </c>
       <c r="Q5" s="10" t="n">
         <v>0.15</v>
@@ -10693,16 +10693,16 @@
         <v>0.36</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>0.64</v>
+        <v>0.59</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>1.19</v>
+        <v>1.11</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.46</v>
+        <v>0.44</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.36</v>
+        <v>0.34</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -10781,10 +10781,10 @@
         <v>-0.7</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -10863,7 +10863,7 @@
         <v>-1.58</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.7</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>-0.15</v>
@@ -13077,13 +13077,13 @@
         <v>0.38</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>0.14</v>
+        <v>0.21</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.12</v>
+        <v>-0.11</v>
       </c>
       <c r="Q6" s="9" t="n">
         <v>0.48</v>
@@ -13165,7 +13165,7 @@
         <v>-0.42</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.19</v>
+        <v>-0.18</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>0.33</v>
@@ -13247,7 +13247,7 @@
         <v>0.65</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.23</v>
+        <v>-0.22</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>0.24</v>
@@ -16817,16 +16817,16 @@
         <v>-0.5</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>-0.47</v>
+        <v>-0.52</v>
       </c>
       <c r="O5" s="10" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="P5" s="10" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="Q5" s="10" t="n">
         <v>-1.02</v>
-      </c>
-      <c r="P5" s="10" t="n">
-        <v>-0.12</v>
-      </c>
-      <c r="Q5" s="10" t="n">
-        <v>-1</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -16905,10 +16905,10 @@
         <v>-1.38</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.06</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>-1.07</v>
+        <v>-1.09</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -16987,10 +16987,10 @@
         <v>0.86</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.12</v>
+        <v>-0.13</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>-0.75</v>
+        <v>-0.77</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -17072,7 +17072,7 @@
         <v>-0.22</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.64</v>
+        <v>-0.65</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -18319,34 +18319,34 @@
         <v>1.88</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>1.28</v>
+        <v>1.58</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>2.06</v>
+        <v>2.55</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0.21</v>
+        <v>0.51</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>0.18</v>
+        <v>0.67</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>-0.23</v>
+        <v>-0.18</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.23</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>0.05</v>
+        <v>0.54</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.14</v>
+        <v>-0.09</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>0.35</v>
+        <v>0.43</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -18357,16 +18357,16 @@
         <v/>
       </c>
       <c r="T8" s="9" t="n">
-        <v>0.91</v>
+        <v>0.87</v>
       </c>
       <c r="U8" s="9" t="n">
         <v>0.86</v>
       </c>
       <c r="V8" s="9" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="W8" s="9" t="n">
-        <v>6.63</v>
+        <v>6.59</v>
       </c>
       <c r="X8" s="9" t="n">
         <v>9.31</v>
@@ -18714,16 +18714,16 @@
         <v>6</v>
       </c>
       <c r="E37" s="19" t="n">
-        <v>-0.75</v>
+        <v>-0.8</v>
       </c>
       <c r="F37" s="19" t="n">
         <v>-0.53</v>
       </c>
       <c r="G37" s="19" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="H37" s="19" t="n">
-        <v>0.84</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="38">
@@ -18742,16 +18742,16 @@
         <v>7</v>
       </c>
       <c r="E38" s="21" t="n">
-        <v>-0.67</v>
+        <v>-0.7</v>
       </c>
       <c r="F38" s="21" t="n">
         <v>-0.59</v>
       </c>
       <c r="G38" s="21" t="n">
-        <v>0.33</v>
+        <v>0.44</v>
       </c>
       <c r="H38" s="21" t="n">
-        <v>0.39</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -19201,16 +19201,16 @@
         <v>0.74</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>-0.38</v>
+        <v>-0.46</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>-0.35</v>
+        <v>-0.41</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>-0.16</v>
+        <v>-0.2</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>0.83</v>
+        <v>0.8</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -19289,10 +19289,10 @@
         <v>-0.15</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.18</v>
+        <v>-0.21</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.5</v>
+        <v>0.48</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -19371,10 +19371,10 @@
         <v>-0.4</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-0.23</v>
+        <v>-0.25</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.28</v>
+        <v>0.26</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -19453,10 +19453,10 @@
         <v>0.14</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.09</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -19535,10 +19535,10 @@
         <v>0.13</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.05</v>
+        <v>-0.06</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.23</v>
+        <v>0.22</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -19617,7 +19617,7 @@
         <v>-1.5</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>-0.36</v>
@@ -20557,16 +20557,16 @@
         <v>0.12</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.86</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>0.93</v>
+        <v>0.88</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>0.22</v>
+        <v>0.2</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -20645,10 +20645,10 @@
         <v>1.25</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>0.27</v>
+        <v>0.24</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.44</v>
+        <v>0.42</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -20727,10 +20727,10 @@
         <v>-0.17</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -20809,10 +20809,10 @@
         <v>-1.63</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>-0.01</v>
+        <v>-0.02</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -20891,10 +20891,10 @@
         <v>-0.42</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.05</v>
+        <v>-0.06</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -21913,16 +21913,16 @@
         <v>0.21</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>-0.86</v>
+        <v>-0.85</v>
       </c>
       <c r="O5" s="10" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.87</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-0.54</v>
+        <v>-0.53</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.6</v>
+        <v>0.62</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -22001,10 +22001,10 @@
         <v>-0.52</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.52</v>
+        <v>-0.51</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.38</v>
+        <v>0.39</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -22077,16 +22077,16 @@
         <v>-0.14</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>1.14</v>
+        <v>1.06</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>-0.37</v>
+        <v>-0.42</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.24</v>
+        <v>-0.25</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -22165,7 +22165,7 @@
         <v>-1.58</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.31</v>
+        <v>-0.32</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>0.08</v>
@@ -22941,16 +22941,16 @@
         <v>-0.9399999999999999</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>-0.91</v>
+        <v>-0.85</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>-0.9</v>
+        <v>-0.89</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>-0.91</v>
+        <v>-0.85</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>-0.9</v>
+        <v>-0.89</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -23029,10 +23029,10 @@
         <v>-0.91</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>-0.78</v>
+        <v>-0.75</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>-0.91</v>
+        <v>-0.9</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -23111,7 +23111,7 @@
         <v>-0.8100000000000001</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.82</v>
+        <v>-0.8</v>
       </c>
       <c r="Q4" s="9" t="n">
         <v>-0.87</v>
@@ -23193,10 +23193,10 @@
         <v>1.56</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-1.06</v>
+        <v>-1.05</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>-0.27</v>
+        <v>-0.26</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -23275,10 +23275,10 @@
         <v>-0.57</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-1.08</v>
+        <v>-1.06</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>-0.33</v>
+        <v>-0.32</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -23357,10 +23357,10 @@
         <v>-0.63</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.91</v>
+        <v>-0.9</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>-0.38</v>
+        <v>-0.37</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -24379,16 +24379,16 @@
         <v>-0.25</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>1.3</v>
+        <v>1.36</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>-1</v>
+        <v>-0.99</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.06</v>
+        <v>-0.05</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -24461,16 +24461,16 @@
         <v>-0.31</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>-0.45</v>
+        <v>-0.53</v>
       </c>
       <c r="O5" s="10" t="n">
-        <v>-0.35</v>
+        <v>-0.4</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-0.09</v>
+        <v>-0.1</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>-0.13</v>
+        <v>-0.14</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -24634,7 +24634,7 @@
         <v>-0.08</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -24713,10 +24713,10 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.05</v>
+        <v>-0.06</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -25832,204 +25832,204 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Shrewsbury Town</t>
+          <t>Barnet</t>
         </is>
       </c>
       <c r="B11" s="8">
-        <f>'Shrewsbury Town'!$E$11</f>
+        <f>'Barnet'!$E$11</f>
         <v/>
       </c>
       <c r="C11" s="10">
-        <f>'Shrewsbury Town'!$E$14</f>
+        <f>'Barnet'!$E$14</f>
         <v/>
       </c>
       <c r="D11" s="10">
-        <f>'Shrewsbury Town'!$E$16</f>
+        <f>'Barnet'!$E$16</f>
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>'Shrewsbury Town'!$E$18</f>
+        <f>'Barnet'!$E$18</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>'Shrewsbury Town'!$E$20</f>
+        <f>'Barnet'!$E$20</f>
         <v/>
       </c>
       <c r="G11" s="10">
-        <f>'Shrewsbury Town'!$E$22</f>
+        <f>'Barnet'!$E$22</f>
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>'Shrewsbury Town'!$E$26</f>
+        <f>'Barnet'!$E$26</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>'Shrewsbury Town'!$E$27</f>
+        <f>'Barnet'!$E$27</f>
         <v/>
       </c>
       <c r="J11" s="10">
-        <f>'Shrewsbury Town'!$E$30</f>
+        <f>'Barnet'!$E$30</f>
         <v/>
       </c>
       <c r="K11" s="10">
-        <f>'Shrewsbury Town'!$E$31</f>
+        <f>'Barnet'!$E$31</f>
         <v/>
       </c>
       <c r="L11" s="10">
-        <f>'Shrewsbury Town'!$E$32</f>
+        <f>'Barnet'!$E$32</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Oldham Athletic</t>
+          <t>Shrewsbury Town</t>
         </is>
       </c>
       <c r="B12" s="6">
-        <f>'Oldham Athletic'!$E$11</f>
+        <f>'Shrewsbury Town'!$E$11</f>
         <v/>
       </c>
       <c r="C12" s="9">
-        <f>'Oldham Athletic'!$E$14</f>
+        <f>'Shrewsbury Town'!$E$14</f>
         <v/>
       </c>
       <c r="D12" s="9">
-        <f>'Oldham Athletic'!$E$16</f>
+        <f>'Shrewsbury Town'!$E$16</f>
         <v/>
       </c>
       <c r="E12" s="9">
-        <f>'Oldham Athletic'!$E$18</f>
+        <f>'Shrewsbury Town'!$E$18</f>
         <v/>
       </c>
       <c r="F12" s="9">
-        <f>'Oldham Athletic'!$E$20</f>
+        <f>'Shrewsbury Town'!$E$20</f>
         <v/>
       </c>
       <c r="G12" s="9">
-        <f>'Oldham Athletic'!$E$22</f>
+        <f>'Shrewsbury Town'!$E$22</f>
         <v/>
       </c>
       <c r="H12" s="9">
-        <f>'Oldham Athletic'!$E$26</f>
+        <f>'Shrewsbury Town'!$E$26</f>
         <v/>
       </c>
       <c r="I12" s="9">
-        <f>'Oldham Athletic'!$E$27</f>
+        <f>'Shrewsbury Town'!$E$27</f>
         <v/>
       </c>
       <c r="J12" s="9">
-        <f>'Oldham Athletic'!$E$30</f>
+        <f>'Shrewsbury Town'!$E$30</f>
         <v/>
       </c>
       <c r="K12" s="9">
-        <f>'Oldham Athletic'!$E$31</f>
+        <f>'Shrewsbury Town'!$E$31</f>
         <v/>
       </c>
       <c r="L12" s="9">
-        <f>'Oldham Athletic'!$E$32</f>
+        <f>'Shrewsbury Town'!$E$32</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Bristol Rvs</t>
+          <t>Oldham Athletic</t>
         </is>
       </c>
       <c r="B13" s="8">
-        <f>'Bristol Rvs'!$E$11</f>
+        <f>'Oldham Athletic'!$E$11</f>
         <v/>
       </c>
       <c r="C13" s="10">
-        <f>'Bristol Rvs'!$E$14</f>
+        <f>'Oldham Athletic'!$E$14</f>
         <v/>
       </c>
       <c r="D13" s="10">
-        <f>'Bristol Rvs'!$E$16</f>
+        <f>'Oldham Athletic'!$E$16</f>
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>'Bristol Rvs'!$E$18</f>
+        <f>'Oldham Athletic'!$E$18</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>'Bristol Rvs'!$E$20</f>
+        <f>'Oldham Athletic'!$E$20</f>
         <v/>
       </c>
       <c r="G13" s="10">
-        <f>'Bristol Rvs'!$E$22</f>
+        <f>'Oldham Athletic'!$E$22</f>
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>'Bristol Rvs'!$E$26</f>
+        <f>'Oldham Athletic'!$E$26</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>'Bristol Rvs'!$E$27</f>
+        <f>'Oldham Athletic'!$E$27</f>
         <v/>
       </c>
       <c r="J13" s="10">
-        <f>'Bristol Rvs'!$E$30</f>
+        <f>'Oldham Athletic'!$E$30</f>
         <v/>
       </c>
       <c r="K13" s="10">
-        <f>'Bristol Rvs'!$E$31</f>
+        <f>'Oldham Athletic'!$E$31</f>
         <v/>
       </c>
       <c r="L13" s="10">
-        <f>'Bristol Rvs'!$E$32</f>
+        <f>'Oldham Athletic'!$E$32</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Barnet</t>
+          <t>Bristol Rvs</t>
         </is>
       </c>
       <c r="B14" s="6">
-        <f>'Barnet'!$E$11</f>
+        <f>'Bristol Rvs'!$E$11</f>
         <v/>
       </c>
       <c r="C14" s="9">
-        <f>'Barnet'!$E$14</f>
+        <f>'Bristol Rvs'!$E$14</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>'Barnet'!$E$16</f>
+        <f>'Bristol Rvs'!$E$16</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>'Barnet'!$E$18</f>
+        <f>'Bristol Rvs'!$E$18</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>'Barnet'!$E$20</f>
+        <f>'Bristol Rvs'!$E$20</f>
         <v/>
       </c>
       <c r="G14" s="9">
-        <f>'Barnet'!$E$22</f>
+        <f>'Bristol Rvs'!$E$22</f>
         <v/>
       </c>
       <c r="H14" s="9">
-        <f>'Barnet'!$E$26</f>
+        <f>'Bristol Rvs'!$E$26</f>
         <v/>
       </c>
       <c r="I14" s="9">
-        <f>'Barnet'!$E$27</f>
+        <f>'Bristol Rvs'!$E$27</f>
         <v/>
       </c>
       <c r="J14" s="9">
-        <f>'Barnet'!$E$30</f>
+        <f>'Bristol Rvs'!$E$30</f>
         <v/>
       </c>
       <c r="K14" s="9">
-        <f>'Barnet'!$E$31</f>
+        <f>'Bristol Rvs'!$E$31</f>
         <v/>
       </c>
       <c r="L14" s="9">
-        <f>'Barnet'!$E$32</f>
+        <f>'Bristol Rvs'!$E$32</f>
         <v/>
       </c>
     </row>
@@ -26189,102 +26189,102 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Colchester United</t>
+          <t>Fleetwood Town</t>
         </is>
       </c>
       <c r="B18" s="6">
-        <f>'Colchester United'!$E$11</f>
+        <f>'Fleetwood Town'!$E$11</f>
         <v/>
       </c>
       <c r="C18" s="9">
-        <f>'Colchester United'!$E$14</f>
+        <f>'Fleetwood Town'!$E$14</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>'Colchester United'!$E$16</f>
+        <f>'Fleetwood Town'!$E$16</f>
         <v/>
       </c>
       <c r="E18" s="9">
-        <f>'Colchester United'!$E$18</f>
+        <f>'Fleetwood Town'!$E$18</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>'Colchester United'!$E$20</f>
+        <f>'Fleetwood Town'!$E$20</f>
         <v/>
       </c>
       <c r="G18" s="9">
-        <f>'Colchester United'!$E$22</f>
+        <f>'Fleetwood Town'!$E$22</f>
         <v/>
       </c>
       <c r="H18" s="9">
-        <f>'Colchester United'!$E$26</f>
+        <f>'Fleetwood Town'!$E$26</f>
         <v/>
       </c>
       <c r="I18" s="9">
-        <f>'Colchester United'!$E$27</f>
+        <f>'Fleetwood Town'!$E$27</f>
         <v/>
       </c>
       <c r="J18" s="9">
-        <f>'Colchester United'!$E$30</f>
+        <f>'Fleetwood Town'!$E$30</f>
         <v/>
       </c>
       <c r="K18" s="9">
-        <f>'Colchester United'!$E$31</f>
+        <f>'Fleetwood Town'!$E$31</f>
         <v/>
       </c>
       <c r="L18" s="9">
-        <f>'Colchester United'!$E$32</f>
+        <f>'Fleetwood Town'!$E$32</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Fleetwood Town</t>
+          <t>Colchester United</t>
         </is>
       </c>
       <c r="B19" s="8">
-        <f>'Fleetwood Town'!$E$11</f>
+        <f>'Colchester United'!$E$11</f>
         <v/>
       </c>
       <c r="C19" s="10">
-        <f>'Fleetwood Town'!$E$14</f>
+        <f>'Colchester United'!$E$14</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>'Fleetwood Town'!$E$16</f>
+        <f>'Colchester United'!$E$16</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>'Fleetwood Town'!$E$18</f>
+        <f>'Colchester United'!$E$18</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>'Fleetwood Town'!$E$20</f>
+        <f>'Colchester United'!$E$20</f>
         <v/>
       </c>
       <c r="G19" s="10">
-        <f>'Fleetwood Town'!$E$22</f>
+        <f>'Colchester United'!$E$22</f>
         <v/>
       </c>
       <c r="H19" s="10">
-        <f>'Fleetwood Town'!$E$26</f>
+        <f>'Colchester United'!$E$26</f>
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>'Fleetwood Town'!$E$27</f>
+        <f>'Colchester United'!$E$27</f>
         <v/>
       </c>
       <c r="J19" s="10">
-        <f>'Fleetwood Town'!$E$30</f>
+        <f>'Colchester United'!$E$30</f>
         <v/>
       </c>
       <c r="K19" s="10">
-        <f>'Fleetwood Town'!$E$31</f>
+        <f>'Colchester United'!$E$31</f>
         <v/>
       </c>
       <c r="L19" s="10">
-        <f>'Fleetwood Town'!$E$32</f>
+        <f>'Colchester United'!$E$32</f>
         <v/>
       </c>
     </row>
@@ -27145,13 +27145,13 @@
         <v>0.32</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>-0.65</v>
+        <v>-0.58</v>
       </c>
       <c r="O5" s="10" t="n">
-        <v>1.7</v>
+        <v>1.71</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-0.55</v>
+        <v>-0.54</v>
       </c>
       <c r="Q5" s="10" t="n">
         <v>0.46</v>
@@ -27227,16 +27227,16 @@
         <v>-0.01</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>-0.65</v>
+        <v>-0.64</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>-0.97</v>
+        <v>-0.91</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.57</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.17</v>
+        <v>0.19</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -27315,10 +27315,10 @@
         <v>-0.45</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.32</v>
+        <v>-0.3</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -27397,10 +27397,10 @@
         <v>-0.85</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.31</v>
+        <v>-0.3</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.06</v>
+        <v>-0.05</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -29857,16 +29857,16 @@
         <v>-0.3</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>1.06</v>
+        <v>1.07</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>0.53</v>
+        <v>0.6</v>
       </c>
       <c r="P7" s="10" t="n">
         <v>0.62</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>-0.5</v>
+        <v>-0.49</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -29948,7 +29948,7 @@
         <v>0.53</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.22</v>
+        <v>-0.21</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -30721,16 +30721,16 @@
         <v>0.2</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>-0.62</v>
+        <v>-0.67</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>0.08</v>
+        <v>-0</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>-0.62</v>
+        <v>-0.67</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>0.08</v>
+        <v>-0</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -30809,10 +30809,10 @@
         <v>0.76</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>-0.91</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>0.42</v>
+        <v>0.38</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -30891,10 +30891,10 @@
         <v>-0.65</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.61</v>
+        <v>-0.63</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.06</v>
+        <v>0.03</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -30973,10 +30973,10 @@
         <v>-0.49</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-0.33</v>
+        <v>-0.34</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>-0.08</v>
+        <v>-0.1</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -31055,10 +31055,10 @@
         <v>-0.04</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.54</v>
+        <v>-0.55</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.09</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -31140,7 +31140,7 @@
         <v>-0.4</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -31195,34 +31195,34 @@
         <v>1.06</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>1.63</v>
+        <v>1.25</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>-0.46</v>
+        <v>-0.83</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>-0.53</v>
+        <v>-0.6</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>0.34</v>
+        <v>0.28</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.39</v>
+        <v>-0.45</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -31233,16 +31233,16 @@
         <v/>
       </c>
       <c r="T8" s="9" t="n">
-        <v>1.68</v>
+        <v>1.46</v>
       </c>
       <c r="U8" s="9" t="n">
         <v>2.04</v>
       </c>
       <c r="V8" s="9" t="n">
-        <v>-0.35</v>
+        <v>-0.58</v>
       </c>
       <c r="W8" s="9" t="n">
-        <v>8.81</v>
+        <v>8.59</v>
       </c>
       <c r="X8" s="9" t="n">
         <v>12.08</v>
@@ -31562,16 +31562,16 @@
         <v>2</v>
       </c>
       <c r="E36" s="19" t="n">
-        <v>-0.77</v>
+        <v>-0.84</v>
       </c>
       <c r="F36" s="19" t="n">
-        <v>-0.78</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="G36" s="19" t="n">
-        <v>-0.52</v>
+        <v>-0.62</v>
       </c>
       <c r="H36" s="19" t="n">
-        <v>-0.33</v>
+        <v>-0.55</v>
       </c>
     </row>
     <row r="37">
@@ -31618,13 +31618,13 @@
         <v>9</v>
       </c>
       <c r="E38" s="21" t="n">
-        <v>-0.7</v>
+        <v>-0.75</v>
       </c>
       <c r="F38" s="21" t="n">
-        <v>-0.58</v>
+        <v>-0.9</v>
       </c>
       <c r="G38" s="21" t="n">
-        <v>-0.28</v>
+        <v>-0.35</v>
       </c>
       <c r="H38" s="21" t="n">
         <v>-0.33</v>
@@ -32077,16 +32077,16 @@
         <v>-0.39</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.51</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>-0.78</v>
+        <v>-0.86</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>0.3</v>
+        <v>0.28</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>-0.46</v>
+        <v>-0.5</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -32159,13 +32159,13 @@
         <v>-0.46</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>-0.65</v>
+        <v>-0.64</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>-0.12</v>
+        <v>-0.06</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.02</v>
+        <v>-0.03</v>
       </c>
       <c r="Q4" s="9" t="n">
         <v>-0.35</v>
@@ -32247,10 +32247,10 @@
         <v>0.08</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-0.05</v>
+        <v>-0.06</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>-0.24</v>
+        <v>-0.25</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -32323,16 +32323,16 @@
         <v>-0.57</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>-0.91</v>
+        <v>-0.99</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-0.74</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.22</v>
+        <v>-0.24</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>-0.33</v>
+        <v>-0.34</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -32411,10 +32411,10 @@
         <v>0.12</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.2</v>
+        <v>-0.22</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>-0.26</v>
+        <v>-0.27</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -32493,10 +32493,10 @@
         <v>-0.48</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.01</v>
+        <v>-0.03</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.31</v>
+        <v>-0.32</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -33743,34 +33743,34 @@
         <v>2.08</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>1.63</v>
+        <v>1.25</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>-0.46</v>
+        <v>-0.83</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>-0.04</v>
+        <v>-0.05</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>0.15</v>
+        <v>0.09</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-0.1</v>
+        <v>-0.16</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>0.04</v>
+        <v>-0.34</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.14</v>
+        <v>-0.15</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>0.21</v>
+        <v>0.14</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -33781,16 +33781,16 @@
         <v/>
       </c>
       <c r="T8" s="9" t="n">
-        <v>1.07</v>
+        <v>1.27</v>
       </c>
       <c r="U8" s="9" t="n">
         <v>0.76</v>
       </c>
       <c r="V8" s="9" t="n">
-        <v>0.32</v>
+        <v>0.51</v>
       </c>
       <c r="W8" s="9" t="n">
-        <v>7.45</v>
+        <v>7.64</v>
       </c>
       <c r="X8" s="9" t="n">
         <v>8.09</v>
@@ -34138,16 +34138,16 @@
         <v>8</v>
       </c>
       <c r="E37" s="19" t="n">
-        <v>-0.73</v>
+        <v>-0.65</v>
       </c>
       <c r="F37" s="19" t="n">
         <v>-0.67</v>
       </c>
       <c r="G37" s="19" t="n">
-        <v>-0.48</v>
+        <v>-0.59</v>
       </c>
       <c r="H37" s="19" t="n">
-        <v>-0.17</v>
+        <v>-0.39</v>
       </c>
     </row>
     <row r="38">
@@ -34166,13 +34166,13 @@
         <v>11</v>
       </c>
       <c r="E38" s="21" t="n">
-        <v>-0.19</v>
+        <v>-0.15</v>
       </c>
       <c r="F38" s="21" t="n">
         <v>-0.19</v>
       </c>
       <c r="G38" s="21" t="n">
-        <v>-0.14</v>
+        <v>-0.21</v>
       </c>
       <c r="H38" s="21" t="n">
         <v>-0.01</v>
@@ -37501,13 +37501,13 @@
         <v>-0.03</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>0.64</v>
+        <v>0.7</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>-0.48</v>
+        <v>-0.47</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>-0.13</v>
@@ -37589,7 +37589,7 @@
         <v>0</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>-0.24</v>
@@ -45876,28 +45876,28 @@
         <v>1.06</v>
       </c>
       <c r="H84" s="9" t="n">
-        <v>1.63</v>
+        <v>1.25</v>
       </c>
       <c r="I84" s="9" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="J84" s="9" t="n">
-        <v>-0.46</v>
+        <v>-0.83</v>
       </c>
       <c r="K84" s="9" t="n">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="L84" s="9" t="n">
-        <v>-0.58</v>
+        <v>-0.9</v>
       </c>
       <c r="M84" s="9" t="n">
-        <v>-0.33</v>
+        <v>-0.77</v>
       </c>
       <c r="N84" s="9" t="n">
-        <v>1.68</v>
+        <v>1.46</v>
       </c>
       <c r="O84" s="9" t="n">
-        <v>1.07</v>
+        <v>1.27</v>
       </c>
       <c r="P84" s="9" t="n">
         <v>2.04</v>
@@ -45935,28 +45935,28 @@
         <v>1.07</v>
       </c>
       <c r="H85" s="10" t="n">
-        <v>2.06</v>
+        <v>2.55</v>
       </c>
       <c r="I85" s="10" t="n">
-        <v>1.28</v>
+        <v>1.58</v>
       </c>
       <c r="J85" s="10" t="n">
-        <v>0.18</v>
+        <v>0.67</v>
       </c>
       <c r="K85" s="10" t="n">
-        <v>0.21</v>
+        <v>0.51</v>
       </c>
       <c r="L85" s="10" t="n">
-        <v>-0.03</v>
+        <v>0.16</v>
       </c>
       <c r="M85" s="10" t="n">
-        <v>0.39</v>
+        <v>1.18</v>
       </c>
       <c r="N85" s="10" t="n">
-        <v>1.87</v>
+        <v>1.95</v>
       </c>
       <c r="O85" s="10" t="n">
-        <v>0.91</v>
+        <v>0.87</v>
       </c>
       <c r="P85" s="10" t="n">
         <v>1.91</v>
@@ -46438,16 +46438,16 @@
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>-0.14</v>
+        <v>-0.11</v>
       </c>
       <c r="C17" s="9" t="n">
-        <v>-0.03</v>
+        <v>0.16</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>0.22</v>
+        <v>0.31</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>-0.52</v>
@@ -46459,51 +46459,51 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Port Vale</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>-0.16</v>
+        <v>-0.15</v>
       </c>
       <c r="C18" s="10" t="n">
-        <v>-0.22</v>
+        <v>-0.19</v>
       </c>
       <c r="D18" s="10" t="n">
-        <v>0.27</v>
+        <v>0.52</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>0.31</v>
+        <v>0.51</v>
       </c>
       <c r="F18" s="10" t="n">
-        <v>-0.49</v>
+        <v>-0.65</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>-0.55</v>
+        <v>-0.67</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Swindon Town</t>
+          <t>Port Vale</t>
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>-0.19</v>
+        <v>-0.16</v>
       </c>
       <c r="C19" s="9" t="n">
-        <v>-0.19</v>
+        <v>-0.22</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>0.52</v>
+        <v>0.27</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>0.51</v>
+        <v>0.31</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>-0.73</v>
+        <v>-0.49</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>-0.67</v>
+        <v>-0.55</v>
       </c>
     </row>
     <row r="20">
@@ -46613,7 +46613,7 @@
         </is>
       </c>
       <c r="B24" s="10" t="n">
-        <v>-0.67</v>
+        <v>-0.7</v>
       </c>
       <c r="C24" s="10" t="n">
         <v>-0.59</v>
@@ -46625,7 +46625,7 @@
         <v>-0.59</v>
       </c>
       <c r="F24" s="10" t="n">
-        <v>-0.75</v>
+        <v>-0.8</v>
       </c>
       <c r="G24" s="10" t="n">
         <v>-0.53</v>
@@ -46638,16 +46638,16 @@
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>-0.7</v>
+        <v>-0.75</v>
       </c>
       <c r="C25" s="9" t="n">
-        <v>-0.58</v>
+        <v>-0.9</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>-0.77</v>
+        <v>-0.84</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>-0.78</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>-0.62</v>
@@ -47103,23 +47103,23 @@
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>Port Vale</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="B45" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="C45" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="D45" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C45" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="D45" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E45" s="8" t="n">
-        <v>1</v>
-      </c>
       <c r="F45" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G45" s="8" t="n">
         <v>8</v>
@@ -47128,23 +47128,23 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Swindon Town</t>
+          <t>Port Vale</t>
         </is>
       </c>
       <c r="B46" s="6" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C46" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F46" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G46" s="6" t="n">
         <v>8</v>
@@ -48061,78 +48061,78 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Port Vale</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="B17" s="14">
-        <f>'Port Vale'!$E$22</f>
+        <f>'Swindon Town'!$E$22</f>
         <v/>
       </c>
       <c r="C17" s="9">
-        <f>'Port Vale'!$R$2</f>
+        <f>'Swindon Town'!$R$2</f>
         <v/>
       </c>
       <c r="D17" s="9">
-        <f>'Port Vale'!$R$3</f>
+        <f>'Swindon Town'!$R$3</f>
         <v/>
       </c>
       <c r="E17" s="9">
-        <f>'Port Vale'!$R$4</f>
+        <f>'Swindon Town'!$R$4</f>
         <v/>
       </c>
       <c r="F17" s="9">
-        <f>'Port Vale'!$R$5</f>
+        <f>'Swindon Town'!$R$5</f>
         <v/>
       </c>
       <c r="G17" s="9">
-        <f>'Port Vale'!$R$6</f>
+        <f>'Swindon Town'!$R$6</f>
         <v/>
       </c>
       <c r="H17" s="9">
-        <f>'Port Vale'!$R$7</f>
+        <f>'Swindon Town'!$R$7</f>
         <v/>
       </c>
       <c r="I17" s="9">
-        <f>'Port Vale'!$R$8</f>
+        <f>'Swindon Town'!$R$8</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Swindon Town</t>
+          <t>Port Vale</t>
         </is>
       </c>
       <c r="B18" s="14">
-        <f>'Swindon Town'!$E$22</f>
+        <f>'Port Vale'!$E$22</f>
         <v/>
       </c>
       <c r="C18" s="9">
-        <f>'Swindon Town'!$R$2</f>
+        <f>'Port Vale'!$R$2</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>'Swindon Town'!$R$3</f>
+        <f>'Port Vale'!$R$3</f>
         <v/>
       </c>
       <c r="E18" s="9">
-        <f>'Swindon Town'!$R$4</f>
+        <f>'Port Vale'!$R$4</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>'Swindon Town'!$R$5</f>
+        <f>'Port Vale'!$R$5</f>
         <v/>
       </c>
       <c r="G18" s="9">
-        <f>'Swindon Town'!$R$6</f>
+        <f>'Port Vale'!$R$6</f>
         <v/>
       </c>
       <c r="H18" s="9">
-        <f>'Swindon Town'!$R$7</f>
+        <f>'Port Vale'!$R$7</f>
         <v/>
       </c>
       <c r="I18" s="9">
-        <f>'Swindon Town'!$R$8</f>
+        <f>'Port Vale'!$R$8</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly League Two data update: 2026-10-06
</commit_message>
<xml_diff>
--- a/data/league-two_xg_report.xlsx
+++ b/data/league-two_xg_report.xlsx
@@ -1172,7 +1172,7 @@
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="5" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1263,51 +1263,51 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Chesterfield</t>
+          <t>Exeter</t>
         </is>
       </c>
       <c r="B4" s="14" t="n">
-        <v>0.79</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>0.38</v>
+        <v>1.11</v>
       </c>
       <c r="D4" s="9" t="n">
-        <v>0.54</v>
+        <v>0.61</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>-0.34</v>
+        <v>1.06</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>1.62</v>
+        <v>-0.44</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>1.73</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Exeter</t>
+          <t>Chesterfield</t>
         </is>
       </c>
       <c r="B5" s="14" t="n">
         <v>0.79</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>1.11</v>
+        <v>0.38</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>0.61</v>
+        <v>0.54</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>1.06</v>
+        <v>-0.34</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>-0.44</v>
+        <v>1.62</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>1.61</v>
+        <v>1.73</v>
       </c>
     </row>
     <row r="6">
@@ -1355,7 +1355,7 @@
         <v>2.44</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>-0.4</v>
+        <v>-0.43</v>
       </c>
     </row>
     <row r="8">
@@ -1637,51 +1637,51 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Crewe Alexandra</t>
+          <t>Salford City</t>
         </is>
       </c>
       <c r="B20" s="14" t="n">
-        <v>-0.62</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>-0.62</v>
+        <v>-2.23</v>
       </c>
       <c r="D20" s="9" t="n">
-        <v>-0.58</v>
+        <v>0.73</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>-1.22</v>
+        <v>-0.98</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>-1.82</v>
+        <v>-0.9</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>1.14</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Salford City</t>
+          <t>Crewe Alexandra</t>
         </is>
       </c>
       <c r="B21" s="14" t="n">
         <v>-0.63</v>
       </c>
       <c r="C21" s="9" t="n">
-        <v>-2.23</v>
+        <v>-0.62</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>0.73</v>
+        <v>-0.58</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>-0.98</v>
+        <v>-1.22</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>-0.9</v>
+        <v>-1.82</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>0.21</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="22">
@@ -1871,7 +1871,7 @@
         <v>1.82</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>0.4</v>
+        <v>0.43</v>
       </c>
     </row>
     <row r="3">
@@ -1927,7 +1927,7 @@
         </is>
       </c>
       <c r="B5" s="14" t="n">
-        <v>0.5</v>
+        <v>0.48</v>
       </c>
       <c r="C5" s="9" t="n">
         <v>1.54</v>
@@ -1942,7 +1942,7 @@
         <v>0.4</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>-1.61</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="6">
@@ -2343,51 +2343,51 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Fleetwood Town</t>
+          <t>Bristol Rvs</t>
         </is>
       </c>
       <c r="B23" s="14" t="n">
-        <v>-0.68</v>
+        <v>-0.71</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>-0.38</v>
+        <v>0.22</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>-0.68</v>
+        <v>0.88</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>-1.97</v>
+        <v>-1.15</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>-0.16</v>
+        <v>-2.38</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>-0.21</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Bristol Rvs</t>
+          <t>Fleetwood Town</t>
         </is>
       </c>
       <c r="B24" s="14" t="n">
-        <v>-0.71</v>
+        <v>-0.75</v>
       </c>
       <c r="C24" s="9" t="n">
-        <v>0.22</v>
+        <v>-0.38</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>0.88</v>
+        <v>-0.68</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>-1.15</v>
+        <v>-1.97</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>-2.38</v>
+        <v>-0.16</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>-1.14</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="25">
@@ -2762,150 +2762,150 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Cheltenham Town</t>
+          <t>Fleetwood Town</t>
         </is>
       </c>
       <c r="B7" s="14">
-        <f>'Cheltenham Town'!$E$26</f>
+        <f>'Fleetwood Town'!$E$26</f>
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>'Cheltenham Town'!$S$2</f>
+        <f>'Fleetwood Town'!$S$2</f>
         <v/>
       </c>
       <c r="D7" s="9">
-        <f>'Cheltenham Town'!$S$3</f>
+        <f>'Fleetwood Town'!$S$3</f>
         <v/>
       </c>
       <c r="E7" s="9">
-        <f>'Cheltenham Town'!$S$4</f>
+        <f>'Fleetwood Town'!$S$4</f>
         <v/>
       </c>
       <c r="F7" s="9">
-        <f>'Cheltenham Town'!$S$5</f>
+        <f>'Fleetwood Town'!$S$5</f>
         <v/>
       </c>
       <c r="G7" s="9">
-        <f>'Cheltenham Town'!$S$6</f>
+        <f>'Fleetwood Town'!$S$6</f>
         <v/>
       </c>
       <c r="H7" s="9">
-        <f>'Cheltenham Town'!$S$7</f>
+        <f>'Fleetwood Town'!$S$7</f>
         <v/>
       </c>
       <c r="I7" s="9">
-        <f>'Cheltenham Town'!$S$8</f>
+        <f>'Fleetwood Town'!$S$8</f>
         <v/>
       </c>
       <c r="J7" s="9">
-        <f>'Cheltenham Town'!$S$9</f>
+        <f>'Fleetwood Town'!$S$9</f>
         <v/>
       </c>
       <c r="K7" s="9">
-        <f>'Cheltenham Town'!$S$10</f>
+        <f>'Fleetwood Town'!$S$10</f>
         <v/>
       </c>
       <c r="L7" s="14">
-        <f>'Cheltenham Town'!$E$27</f>
+        <f>'Fleetwood Town'!$E$27</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>York</t>
+          <t>Cheltenham Town</t>
         </is>
       </c>
       <c r="B8" s="14">
-        <f>'York'!$E$25</f>
+        <f>'Cheltenham Town'!$E$26</f>
         <v/>
       </c>
       <c r="C8" s="9">
-        <f>'York'!$S$2</f>
+        <f>'Cheltenham Town'!$S$2</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>'York'!$S$3</f>
+        <f>'Cheltenham Town'!$S$3</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>'York'!$S$4</f>
+        <f>'Cheltenham Town'!$S$4</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>'York'!$S$5</f>
+        <f>'Cheltenham Town'!$S$5</f>
         <v/>
       </c>
       <c r="G8" s="9">
-        <f>'York'!$S$6</f>
+        <f>'Cheltenham Town'!$S$6</f>
         <v/>
       </c>
       <c r="H8" s="9">
-        <f>'York'!$S$7</f>
+        <f>'Cheltenham Town'!$S$7</f>
         <v/>
       </c>
       <c r="I8" s="9">
-        <f>'York'!$S$8</f>
+        <f>'Cheltenham Town'!$S$8</f>
         <v/>
       </c>
       <c r="J8" s="9">
-        <f>'York'!$S$9</f>
-        <v/>
-      </c>
-      <c r="K8" s="6" t="n"/>
+        <f>'Cheltenham Town'!$S$9</f>
+        <v/>
+      </c>
+      <c r="K8" s="9">
+        <f>'Cheltenham Town'!$S$10</f>
+        <v/>
+      </c>
       <c r="L8" s="14">
-        <f>'York'!$E$26</f>
+        <f>'Cheltenham Town'!$E$27</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Fleetwood Town</t>
+          <t>York</t>
         </is>
       </c>
       <c r="B9" s="14">
-        <f>'Fleetwood Town'!$E$26</f>
+        <f>'York'!$E$25</f>
         <v/>
       </c>
       <c r="C9" s="9">
-        <f>'Fleetwood Town'!$S$2</f>
+        <f>'York'!$S$2</f>
         <v/>
       </c>
       <c r="D9" s="9">
-        <f>'Fleetwood Town'!$S$3</f>
+        <f>'York'!$S$3</f>
         <v/>
       </c>
       <c r="E9" s="9">
-        <f>'Fleetwood Town'!$S$4</f>
+        <f>'York'!$S$4</f>
         <v/>
       </c>
       <c r="F9" s="9">
-        <f>'Fleetwood Town'!$S$5</f>
+        <f>'York'!$S$5</f>
         <v/>
       </c>
       <c r="G9" s="9">
-        <f>'Fleetwood Town'!$S$6</f>
+        <f>'York'!$S$6</f>
         <v/>
       </c>
       <c r="H9" s="9">
-        <f>'Fleetwood Town'!$S$7</f>
+        <f>'York'!$S$7</f>
         <v/>
       </c>
       <c r="I9" s="9">
-        <f>'Fleetwood Town'!$S$8</f>
+        <f>'York'!$S$8</f>
         <v/>
       </c>
       <c r="J9" s="9">
-        <f>'Fleetwood Town'!$S$9</f>
-        <v/>
-      </c>
-      <c r="K9" s="9">
-        <f>'Fleetwood Town'!$S$10</f>
-        <v/>
-      </c>
+        <f>'York'!$S$9</f>
+        <v/>
+      </c>
+      <c r="K9" s="6" t="n"/>
       <c r="L9" s="14">
-        <f>'Fleetwood Town'!$E$27</f>
+        <f>'York'!$E$26</f>
         <v/>
       </c>
     </row>
@@ -3464,102 +3464,102 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Salford City</t>
         </is>
       </c>
       <c r="B21" s="14">
-        <f>'Newport County'!$E$26</f>
+        <f>'Salford City'!$E$26</f>
         <v/>
       </c>
       <c r="C21" s="9">
-        <f>'Newport County'!$S$2</f>
+        <f>'Salford City'!$S$2</f>
         <v/>
       </c>
       <c r="D21" s="9">
-        <f>'Newport County'!$S$3</f>
+        <f>'Salford City'!$S$3</f>
         <v/>
       </c>
       <c r="E21" s="9">
-        <f>'Newport County'!$S$4</f>
+        <f>'Salford City'!$S$4</f>
         <v/>
       </c>
       <c r="F21" s="9">
-        <f>'Newport County'!$S$5</f>
+        <f>'Salford City'!$S$5</f>
         <v/>
       </c>
       <c r="G21" s="9">
-        <f>'Newport County'!$S$6</f>
+        <f>'Salford City'!$S$6</f>
         <v/>
       </c>
       <c r="H21" s="9">
-        <f>'Newport County'!$S$7</f>
+        <f>'Salford City'!$S$7</f>
         <v/>
       </c>
       <c r="I21" s="9">
-        <f>'Newport County'!$S$8</f>
+        <f>'Salford City'!$S$8</f>
         <v/>
       </c>
       <c r="J21" s="9">
-        <f>'Newport County'!$S$9</f>
+        <f>'Salford City'!$S$9</f>
         <v/>
       </c>
       <c r="K21" s="9">
-        <f>'Newport County'!$S$10</f>
+        <f>'Salford City'!$S$10</f>
         <v/>
       </c>
       <c r="L21" s="14">
-        <f>'Newport County'!$E$27</f>
+        <f>'Salford City'!$E$27</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Salford City</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="B22" s="14">
-        <f>'Salford City'!$E$26</f>
+        <f>'Newport County'!$E$26</f>
         <v/>
       </c>
       <c r="C22" s="9">
-        <f>'Salford City'!$S$2</f>
+        <f>'Newport County'!$S$2</f>
         <v/>
       </c>
       <c r="D22" s="9">
-        <f>'Salford City'!$S$3</f>
+        <f>'Newport County'!$S$3</f>
         <v/>
       </c>
       <c r="E22" s="9">
-        <f>'Salford City'!$S$4</f>
+        <f>'Newport County'!$S$4</f>
         <v/>
       </c>
       <c r="F22" s="9">
-        <f>'Salford City'!$S$5</f>
+        <f>'Newport County'!$S$5</f>
         <v/>
       </c>
       <c r="G22" s="9">
-        <f>'Salford City'!$S$6</f>
+        <f>'Newport County'!$S$6</f>
         <v/>
       </c>
       <c r="H22" s="9">
-        <f>'Salford City'!$S$7</f>
+        <f>'Newport County'!$S$7</f>
         <v/>
       </c>
       <c r="I22" s="9">
-        <f>'Salford City'!$S$8</f>
+        <f>'Newport County'!$S$8</f>
         <v/>
       </c>
       <c r="J22" s="9">
-        <f>'Salford City'!$S$9</f>
+        <f>'Newport County'!$S$9</f>
         <v/>
       </c>
       <c r="K22" s="9">
-        <f>'Salford City'!$S$10</f>
+        <f>'Newport County'!$S$10</f>
         <v/>
       </c>
       <c r="L22" s="14">
-        <f>'Salford City'!$E$27</f>
+        <f>'Newport County'!$E$27</f>
         <v/>
       </c>
     </row>
@@ -5058,25 +5058,25 @@
         <v>0.85</v>
       </c>
       <c r="E3" s="10" t="n">
-        <v>-0.49</v>
+        <v>-0.45</v>
       </c>
       <c r="F3" s="10" t="n">
-        <v>-0.62</v>
+        <v>-0.66</v>
       </c>
       <c r="G3" s="10" t="n">
-        <v>0.98</v>
+        <v>1.06</v>
       </c>
       <c r="H3" s="10" t="n">
         <v>2.87</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>-0.38</v>
+        <v>-0.3</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>0.27</v>
+        <v>0.35</v>
       </c>
       <c r="K3" s="10" t="n">
-        <v>2.76</v>
+        <v>2.92</v>
       </c>
       <c r="L3" s="8" t="inlineStr"/>
     </row>
@@ -5142,13 +5142,13 @@
         <v>0.86</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="F5" s="10" t="n">
         <v>0.65</v>
       </c>
       <c r="G5" s="10" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="H5" s="10" t="n">
         <v>2.83</v>
@@ -5157,10 +5157,10 @@
         <v>0.49</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>-0.29</v>
+        <v>-0.28</v>
       </c>
       <c r="K5" s="10" t="n">
-        <v>3.03</v>
+        <v>3.04</v>
       </c>
       <c r="L5" s="8" t="inlineStr"/>
     </row>
@@ -5226,25 +5226,25 @@
         <v>0.01</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>0.47</v>
+        <v>0.46</v>
       </c>
       <c r="G7" s="10" t="n">
-        <v>-0.13</v>
+        <v>-0.11</v>
       </c>
       <c r="H7" s="10" t="n">
         <v>2.66</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>-0.43</v>
+        <v>-0.42</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>-0.03</v>
+        <v>-0.02</v>
       </c>
       <c r="K7" s="10" t="n">
-        <v>2.2</v>
+        <v>2.22</v>
       </c>
       <c r="L7" s="8" t="inlineStr"/>
     </row>
@@ -5310,13 +5310,13 @@
         <v>-0.29</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>-0.17</v>
+        <v>-0.18</v>
       </c>
       <c r="F9" s="10" t="n">
         <v>0.04</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>-0.5</v>
+        <v>-0.51</v>
       </c>
       <c r="H9" s="10" t="n">
         <v>2.78</v>
@@ -5325,10 +5325,10 @@
         <v>-0.27</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="K9" s="10" t="n">
-        <v>2.61</v>
+        <v>2.62</v>
       </c>
       <c r="L9" s="8" t="inlineStr"/>
     </row>
@@ -5654,13 +5654,13 @@
         <v>-0</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>0.88</v>
+        <v>0.86</v>
       </c>
       <c r="P3" s="10" t="n">
         <v>0.7</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -5742,7 +5742,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.35</v>
+        <v>0.34</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -5824,7 +5824,7 @@
         <v>1.1</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -7007,16 +7007,16 @@
         <v>-0.26</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>0.2</v>
+        <v>0.13</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>0.2</v>
+        <v>0.13</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -7092,13 +7092,13 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>0.65</v>
+        <v>0.64</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>0.42</v>
+        <v>0.39</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -7180,7 +7180,7 @@
         <v>0.04</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -7256,13 +7256,13 @@
         <v>-0.4</v>
       </c>
       <c r="O5" s="10" t="n">
-        <v>-0.09</v>
+        <v>-0.1</v>
       </c>
       <c r="P5" s="10" t="n">
         <v>-0.07000000000000001</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.43</v>
+        <v>0.41</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -7341,10 +7341,10 @@
         <v>0.11</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.22</v>
+        <v>0.21</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.37</v>
+        <v>0.35</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -7426,7 +7426,7 @@
         <v>0.23</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -7499,13 +7499,13 @@
         <v>0.41</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>0.25</v>
+        <v>0.19</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>0.78</v>
+        <v>0.75</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>0.24</v>
@@ -8609,7 +8609,7 @@
         <v>-0.18</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>-0.92</v>
+        <v>-0.93</v>
       </c>
       <c r="O6" s="9" t="n">
         <v>-0.8100000000000001</v>
@@ -8858,10 +8858,10 @@
         <v>0.7</v>
       </c>
       <c r="O9" s="10" t="n">
-        <v>-0.33</v>
+        <v>-0.34</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>-0.26</v>
+        <v>-0.27</v>
       </c>
       <c r="Q9" s="10" t="n">
         <v>-0.2</v>
@@ -8919,16 +8919,16 @@
         <v>1.24</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.74</v>
+        <v>0.79</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>1.59</v>
+        <v>1.6</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>-0.79</v>
+        <v>-0.74</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="L10" s="9" t="n">
         <v>-0.45</v>
@@ -8937,13 +8937,13 @@
         <v>0.08</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>-0.84</v>
+        <v>-0.79</v>
       </c>
       <c r="O10" s="9" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>-0.43</v>
+        <v>-0.42</v>
       </c>
       <c r="Q10" s="9" t="n">
         <v>0.04</v>
@@ -8957,16 +8957,16 @@
         <v/>
       </c>
       <c r="T10" s="9" t="n">
-        <v>0.77</v>
+        <v>0.8</v>
       </c>
       <c r="U10" s="9" t="n">
         <v>1.57</v>
       </c>
       <c r="V10" s="9" t="n">
-        <v>-0.8</v>
+        <v>-0.77</v>
       </c>
       <c r="W10" s="9" t="n">
-        <v>14.08</v>
+        <v>14.12</v>
       </c>
       <c r="X10" s="9" t="n">
         <v>14.93</v>
@@ -9317,10 +9317,10 @@
         <v>-0.71</v>
       </c>
       <c r="F39" s="19" t="n">
-        <v>-1.14</v>
+        <v>-1.1</v>
       </c>
       <c r="G39" s="19" t="n">
-        <v>-0.06</v>
+        <v>-0.05</v>
       </c>
       <c r="H39" s="19" t="n">
         <v>0.05</v>
@@ -9348,7 +9348,7 @@
         <v>0.22</v>
       </c>
       <c r="G40" s="21" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="H40" s="21" t="n">
         <v>0.05</v>
@@ -9719,13 +9719,13 @@
         <v>0.84</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>-0.51</v>
+        <v>-0.52</v>
       </c>
       <c r="O2" s="9" t="n">
         <v>0.6899999999999999</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>-0.51</v>
+        <v>-0.52</v>
       </c>
       <c r="Q2" s="9" t="n">
         <v>0.6899999999999999</v>
@@ -11157,16 +11157,16 @@
         <v>0.16</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>0.1</v>
+        <v>0.03</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>0.38</v>
+        <v>0.35</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>0.1</v>
+        <v>0.03</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>0.38</v>
+        <v>0.35</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -11239,16 +11239,16 @@
         <v>-0.41</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>-0.61</v>
+        <v>-0.68</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>0.72</v>
+        <v>0.68</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>-0.12</v>
+        <v>-0.16</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -11321,16 +11321,16 @@
         <v>0.31</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>-0.08</v>
+        <v>-0.1</v>
       </c>
       <c r="O4" s="9" t="n">
         <v>1.72</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>0.45</v>
+        <v>0.42</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.49</v>
+        <v>0.46</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -11409,10 +11409,10 @@
         <v>-0.29</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>0.44</v>
+        <v>0.41</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.3</v>
+        <v>0.27</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -11491,10 +11491,10 @@
         <v>1.11</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.47</v>
+        <v>0.45</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.46</v>
+        <v>0.44</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -11573,10 +11573,10 @@
         <v>-0.61</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.59</v>
+        <v>0.57</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -11658,7 +11658,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.03</v>
+        <v>-0.05</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -14115,13 +14115,13 @@
         <v>0.22</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>-0.26</v>
+        <v>-0.27</v>
       </c>
       <c r="O7" s="10" t="n">
         <v>-0.38</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.09</v>
+        <v>-0.1</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>0.29</v>
@@ -14282,7 +14282,7 @@
         <v>0.75</v>
       </c>
       <c r="O9" s="10" t="n">
-        <v>-0.13</v>
+        <v>-0.14</v>
       </c>
       <c r="P9" s="10" t="n">
         <v>-0.25</v>
@@ -15061,13 +15061,13 @@
         <v>0.91</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>-0.4</v>
+        <v>-0.41</v>
       </c>
       <c r="O2" s="9" t="n">
         <v>1.27</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>-0.4</v>
+        <v>-0.41</v>
       </c>
       <c r="Q2" s="9" t="n">
         <v>1.27</v>
@@ -15149,7 +15149,7 @@
         <v>-0.65</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="Q3" s="10" t="n">
         <v>0.31</v>
@@ -15228,10 +15228,10 @@
         <v>-0.5</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>0.44</v>
+        <v>0.43</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="Q4" s="9" t="n">
         <v>0.35</v>
@@ -15398,7 +15398,7 @@
         <v>0.49</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -15553,7 +15553,7 @@
         <v>0.23</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-0.2</v>
+        <v>-0.21</v>
       </c>
       <c r="O8" s="9" t="n">
         <v>2.24</v>
@@ -16909,7 +16909,7 @@
         <v>0.19</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>-0.76</v>
+        <v>-0.77</v>
       </c>
       <c r="O9" s="10" t="n">
         <v>-1.36</v>
@@ -16973,34 +16973,34 @@
         <v>1.53</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>1.59</v>
+        <v>1.6</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>0.74</v>
+        <v>0.79</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>-0.79</v>
+        <v>-0.74</v>
       </c>
       <c r="L10" s="9" t="n">
         <v>-0.32</v>
       </c>
       <c r="M10" s="9" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>0.36</v>
+        <v>0.37</v>
       </c>
       <c r="O10" s="9" t="n">
-        <v>-0.97</v>
+        <v>-0.92</v>
       </c>
       <c r="P10" s="9" t="n">
         <v>-0.28</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>-0.01</v>
+        <v>-0</v>
       </c>
       <c r="R10" s="9">
         <f>(H10-I10)-(F10-G10)</f>
@@ -17011,16 +17011,16 @@
         <v/>
       </c>
       <c r="T10" s="9" t="n">
-        <v>1.98</v>
+        <v>1.95</v>
       </c>
       <c r="U10" s="9" t="n">
         <v>1.18</v>
       </c>
       <c r="V10" s="9" t="n">
-        <v>0.8</v>
+        <v>0.77</v>
       </c>
       <c r="W10" s="9" t="n">
-        <v>10.89</v>
+        <v>10.86</v>
       </c>
       <c r="X10" s="9" t="n">
         <v>12.08</v>
@@ -17340,13 +17340,13 @@
         <v>5</v>
       </c>
       <c r="E38" s="19" t="n">
-        <v>-0.62</v>
+        <v>-0.63</v>
       </c>
       <c r="F38" s="19" t="n">
         <v>-0.62</v>
       </c>
       <c r="G38" s="19" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="H38" s="19" t="n">
         <v>0.52</v>
@@ -17396,7 +17396,7 @@
         <v>7</v>
       </c>
       <c r="E40" s="21" t="n">
-        <v>-0.17</v>
+        <v>-0.18</v>
       </c>
       <c r="F40" s="21" t="n">
         <v>-0.28</v>
@@ -17405,7 +17405,7 @@
         <v>-0.27</v>
       </c>
       <c r="H40" s="21" t="n">
-        <v>-0.44</v>
+        <v>-0.39</v>
       </c>
     </row>
   </sheetData>
@@ -18411,31 +18411,31 @@
         <v>1.32</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>2.09</v>
+        <v>2.18</v>
       </c>
       <c r="I10" s="9" t="n">
         <v>0.47</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>0.76</v>
+        <v>0.85</v>
       </c>
       <c r="K10" s="9" t="n">
         <v>-0.85</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>-0.14</v>
+        <v>-0.12</v>
       </c>
       <c r="M10" s="9" t="n">
         <v>-0.36</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>1.14</v>
+        <v>1.23</v>
       </c>
       <c r="O10" s="9" t="n">
         <v>-1.21</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>-0.2</v>
+        <v>-0.19</v>
       </c>
       <c r="Q10" s="9" t="n">
         <v>-0.46</v>
@@ -18449,16 +18449,16 @@
         <v/>
       </c>
       <c r="T10" s="9" t="n">
-        <v>2.44</v>
+        <v>2.47</v>
       </c>
       <c r="U10" s="9" t="n">
         <v>1.37</v>
       </c>
       <c r="V10" s="9" t="n">
-        <v>1.06</v>
+        <v>1.1</v>
       </c>
       <c r="W10" s="9" t="n">
-        <v>12.61</v>
+        <v>12.64</v>
       </c>
       <c r="X10" s="9" t="n">
         <v>10.75</v>
@@ -18778,13 +18778,13 @@
         <v>1</v>
       </c>
       <c r="E38" s="19" t="n">
-        <v>0.79</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F38" s="19" t="n">
         <v>1.06</v>
       </c>
       <c r="G38" s="19" t="n">
-        <v>-0.49</v>
+        <v>-0.47</v>
       </c>
       <c r="H38" s="19" t="n">
         <v>-0.84</v>
@@ -18834,13 +18834,13 @@
         <v>6</v>
       </c>
       <c r="E40" s="21" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="F40" s="21" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="G40" s="21" t="n">
-        <v>-0.43</v>
+        <v>-0.42</v>
       </c>
       <c r="H40" s="21" t="n">
         <v>-0.54</v>
@@ -19542,10 +19542,10 @@
         <v>-0.33</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>-0.51</v>
+        <v>-0.52</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.1</v>
+        <v>-0.11</v>
       </c>
       <c r="Q6" s="9" t="n">
         <v>0.11</v>
@@ -19849,34 +19849,34 @@
         <v>1.86</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.45</v>
+        <v>0.62</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>1.51</v>
+        <v>2.04</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.39</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>-0.35</v>
+        <v>0.18</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>-0.32</v>
+        <v>-0.29</v>
       </c>
       <c r="M10" s="9" t="n">
-        <v>0.33</v>
+        <v>0.42</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-0.52</v>
       </c>
       <c r="O10" s="9" t="n">
-        <v>0.1</v>
+        <v>0.63</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>-0.33</v>
+        <v>-0.3</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>0.47</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="R10" s="9">
         <f>(H10-I10)-(F10-G10)</f>
@@ -19887,16 +19887,16 @@
         <v/>
       </c>
       <c r="T10" s="9" t="n">
-        <v>0.58</v>
+        <v>0.5</v>
       </c>
       <c r="U10" s="9" t="n">
         <v>0.83</v>
       </c>
       <c r="V10" s="9" t="n">
-        <v>-0.25</v>
+        <v>-0.34</v>
       </c>
       <c r="W10" s="9" t="n">
-        <v>8.630000000000001</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="X10" s="9" t="n">
         <v>11.94</v>
@@ -20244,13 +20244,13 @@
         <v>7</v>
       </c>
       <c r="E39" s="19" t="n">
-        <v>-0.68</v>
+        <v>-0.75</v>
       </c>
       <c r="F39" s="19" t="n">
-        <v>-0.38</v>
+        <v>-0.57</v>
       </c>
       <c r="G39" s="19" t="n">
-        <v>0.78</v>
+        <v>0.92</v>
       </c>
       <c r="H39" s="19" t="n">
         <v>0.99</v>
@@ -20272,13 +20272,13 @@
         <v>10</v>
       </c>
       <c r="E40" s="21" t="n">
-        <v>-0.62</v>
+        <v>-0.66</v>
       </c>
       <c r="F40" s="21" t="n">
-        <v>-0.49</v>
+        <v>-0.57</v>
       </c>
       <c r="G40" s="21" t="n">
-        <v>0.27</v>
+        <v>0.35</v>
       </c>
       <c r="H40" s="21" t="n">
         <v>0.23</v>
@@ -20731,16 +20731,16 @@
         <v>0.74</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>-0.3</v>
+        <v>-0.37</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>-0.34</v>
+        <v>-0.36</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>-0.18</v>
+        <v>-0.22</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>0.87</v>
+        <v>0.86</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -20819,10 +20819,10 @@
         <v>-0.15</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.2</v>
+        <v>-0.23</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.53</v>
+        <v>0.52</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -20901,10 +20901,10 @@
         <v>-0.51</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-0.21</v>
+        <v>-0.23</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -20983,10 +20983,10 @@
         <v>-0.13</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.03</v>
+        <v>-0.04</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -21065,10 +21065,10 @@
         <v>0.05</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.02</v>
+        <v>-0.03</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -21144,13 +21144,13 @@
         <v>1.38</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>-1.34</v>
+        <v>-1.35</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.22</v>
+        <v>0.21</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.4</v>
+        <v>-0.41</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -21311,7 +21311,7 @@
         <v>0.2</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q10" s="9" t="n">
         <v>-0.32</v>
@@ -22090,13 +22090,13 @@
         <v>0.12</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>-0.25</v>
+        <v>-0.26</v>
       </c>
       <c r="P2" s="9" t="n">
         <v>0.12</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>-0.25</v>
+        <v>-0.26</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -22178,7 +22178,7 @@
         <v>-0.21</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>-0.2</v>
+        <v>-0.21</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -22251,16 +22251,16 @@
         <v>0.12</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>0.97</v>
+        <v>0.91</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>0.9</v>
+        <v>0.88</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -22339,10 +22339,10 @@
         <v>1.15</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>0.27</v>
+        <v>0.25</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.41</v>
+        <v>0.4</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -22421,7 +22421,7 @@
         <v>0.12</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="Q6" s="9" t="n">
         <v>0.35</v>
@@ -22500,10 +22500,10 @@
         <v>-0.13</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>-1.46</v>
+        <v>-1.47</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>0.05</v>
@@ -22585,7 +22585,7 @@
         <v>-0.42</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.47</v>
+        <v>0.46</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>0.02</v>
@@ -22667,7 +22667,7 @@
         <v>0.26</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="Q9" s="10" t="n">
         <v>0.09</v>
@@ -22728,13 +22728,13 @@
         <v>1.56</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>1.1</v>
+        <v>1.13</v>
       </c>
       <c r="J10" s="9" t="n">
         <v>-0.28</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="L10" s="9" t="n">
         <v>0.46</v>
@@ -22746,7 +22746,7 @@
         <v>0.21</v>
       </c>
       <c r="O10" s="9" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.04</v>
       </c>
       <c r="P10" s="9" t="n">
         <v>0.54</v>
@@ -22763,16 +22763,16 @@
         <v/>
       </c>
       <c r="T10" s="9" t="n">
-        <v>1.69</v>
+        <v>1.67</v>
       </c>
       <c r="U10" s="9" t="n">
         <v>1.95</v>
       </c>
       <c r="V10" s="9" t="n">
-        <v>-0.26</v>
+        <v>-0.28</v>
       </c>
       <c r="W10" s="9" t="n">
-        <v>16.63</v>
+        <v>16.61</v>
       </c>
       <c r="X10" s="9" t="n">
         <v>15.97</v>
@@ -23098,10 +23098,10 @@
         <v>0.68</v>
       </c>
       <c r="G38" s="19" t="n">
-        <v>0.44</v>
+        <v>0.45</v>
       </c>
       <c r="H38" s="19" t="n">
-        <v>-0.17</v>
+        <v>-0.14</v>
       </c>
     </row>
     <row r="39">
@@ -23148,7 +23148,7 @@
         <v>10</v>
       </c>
       <c r="E40" s="21" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="F40" s="21" t="n">
         <v>0</v>
@@ -23771,16 +23771,16 @@
         <v>0.21</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>-0.65</v>
+        <v>-0.67</v>
       </c>
       <c r="O5" s="10" t="n">
-        <v>0.71</v>
+        <v>0.65</v>
       </c>
       <c r="P5" s="10" t="n">
         <v>-0.45</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.51</v>
+        <v>0.49</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -23859,10 +23859,10 @@
         <v>-0.52</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.44</v>
+        <v>-0.45</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -23935,16 +23935,16 @@
         <v>-0.14</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>1.16</v>
+        <v>1.09</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>-0.35</v>
+        <v>-0.37</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.18</v>
+        <v>-0.19</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -24023,10 +24023,10 @@
         <v>-1.58</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.25</v>
+        <v>-0.26</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -24105,10 +24105,10 @@
         <v>-0.11</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>-0.17</v>
+        <v>-0.19</v>
       </c>
       <c r="Q9" s="10" t="n">
-        <v>-0.35</v>
+        <v>-0.37</v>
       </c>
       <c r="R9" s="10">
         <f>(H9-I9)-(F9-G9)</f>
@@ -24187,10 +24187,10 @@
         <v>-1.4</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>-0.06</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>-0.54</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="R10" s="9">
         <f>(H10-I10)-(F10-G10)</f>
@@ -25133,7 +25133,7 @@
         <v>-0.46</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.72</v>
+        <v>-0.73</v>
       </c>
       <c r="Q4" s="9" t="n">
         <v>-0.74</v>
@@ -25455,13 +25455,13 @@
         <v>-0.1</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-0.06</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="O8" s="9" t="n">
         <v>-0.14</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.73</v>
+        <v>-0.74</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>-0.18</v>
@@ -26483,16 +26483,16 @@
         <v>-0.31</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>-0.37</v>
+        <v>-0.44</v>
       </c>
       <c r="O5" s="10" t="n">
-        <v>-0.33</v>
+        <v>-0.35</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-0.05</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>-0.14</v>
+        <v>-0.15</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -26571,7 +26571,7 @@
         <v>0.97</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="Q6" s="9" t="n">
         <v>0.08</v>
@@ -26653,7 +26653,7 @@
         <v>0.4</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.04</v>
+        <v>-0.05</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>0.13</v>
@@ -26735,7 +26735,7 @@
         <v>-0.2</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.01</v>
+        <v>-0</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>0.18</v>
@@ -26811,16 +26811,16 @@
         <v>-0.01</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>-0.48</v>
+        <v>-0.5</v>
       </c>
       <c r="O9" s="10" t="n">
-        <v>0.78</v>
+        <v>0.72</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="Q9" s="10" t="n">
-        <v>0.11</v>
+        <v>0.09</v>
       </c>
       <c r="R9" s="10">
         <f>(H9-I9)-(F9-G9)</f>
@@ -29167,7 +29167,7 @@
         <v>-0.01</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>-0.43</v>
+        <v>-0.44</v>
       </c>
       <c r="O4" s="9" t="n">
         <v>0.24</v>
@@ -29331,16 +29331,16 @@
         <v>-0.01</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>-0.45</v>
+        <v>-0.47</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>-1</v>
+        <v>-1.07</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.48</v>
+        <v>-0.49</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -29416,13 +29416,13 @@
         <v>0.91</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>-0.52</v>
+        <v>-0.53</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.25</v>
+        <v>-0.26</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -29504,7 +29504,7 @@
         <v>-0.26</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.09</v>
+        <v>-0.1</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -30526,7 +30526,7 @@
         <v>-0.27</v>
       </c>
       <c r="O5" s="10" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="P5" s="10" t="n">
         <v>-0.93</v>
@@ -30851,16 +30851,16 @@
         <v>0.24</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>-0.1</v>
+        <v>-0.16</v>
       </c>
       <c r="O9" s="10" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.57</v>
       </c>
       <c r="Q9" s="10" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="R9" s="10">
         <f>(H9-I9)-(F9-G9)</f>
@@ -30939,7 +30939,7 @@
         <v>-0.21</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>-0.4</v>
+        <v>-0.41</v>
       </c>
       <c r="Q10" s="9" t="n">
         <v>0.25</v>
@@ -32046,7 +32046,7 @@
         <v>-0.6</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>-1.28</v>
+        <v>-1.29</v>
       </c>
       <c r="P6" s="9" t="n">
         <v>0.5</v>
@@ -32125,16 +32125,16 @@
         <v>-0.3</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>1.2</v>
+        <v>1.18</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>0.45</v>
+        <v>0.38</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.62</v>
+        <v>0.61</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>-0.45</v>
+        <v>-0.46</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -32216,7 +32216,7 @@
         <v>0.57</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.22</v>
+        <v>-0.24</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -32289,16 +32289,16 @@
         <v>-0.5600000000000001</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>-1.05</v>
+        <v>-1.06</v>
       </c>
       <c r="O9" s="10" t="n">
         <v>-0.79</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>0.46</v>
+        <v>0.45</v>
       </c>
       <c r="Q9" s="10" t="n">
-        <v>-0.49</v>
+        <v>-0.5</v>
       </c>
       <c r="R9" s="10">
         <f>(H9-I9)-(F9-G9)</f>
@@ -32356,25 +32356,25 @@
         <v>0.47</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>2.09</v>
+        <v>2.18</v>
       </c>
       <c r="J10" s="9" t="n">
         <v>-0.85</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>0.76</v>
+        <v>0.85</v>
       </c>
       <c r="L10" s="9" t="n">
         <v>-0.04</v>
       </c>
       <c r="M10" s="9" t="n">
-        <v>-0.37</v>
+        <v>-0.36</v>
       </c>
       <c r="N10" s="9" t="n">
         <v>-0.53</v>
       </c>
       <c r="O10" s="9" t="n">
-        <v>0.91</v>
+        <v>1</v>
       </c>
       <c r="P10" s="9" t="n">
         <v>0.03</v>
@@ -32391,16 +32391,16 @@
         <v/>
       </c>
       <c r="T10" s="9" t="n">
-        <v>0.39</v>
+        <v>0.36</v>
       </c>
       <c r="U10" s="9" t="n">
         <v>1.36</v>
       </c>
       <c r="V10" s="9" t="n">
-        <v>-0.98</v>
+        <v>-1</v>
       </c>
       <c r="W10" s="9" t="n">
-        <v>14.21</v>
+        <v>14.19</v>
       </c>
       <c r="X10" s="9" t="n">
         <v>11.59</v>
@@ -32748,16 +32748,16 @@
         <v>6</v>
       </c>
       <c r="E39" s="19" t="n">
-        <v>0.5</v>
+        <v>0.48</v>
       </c>
       <c r="F39" s="19" t="n">
         <v>0.57</v>
       </c>
       <c r="G39" s="19" t="n">
-        <v>-0.3</v>
+        <v>-0.28</v>
       </c>
       <c r="H39" s="19" t="n">
-        <v>-0.1</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="40">
@@ -32776,13 +32776,13 @@
         <v>12</v>
       </c>
       <c r="E40" s="21" t="n">
-        <v>0.47</v>
+        <v>0.46</v>
       </c>
       <c r="F40" s="21" t="n">
         <v>0.57</v>
       </c>
       <c r="G40" s="21" t="n">
-        <v>-0.03</v>
+        <v>-0.02</v>
       </c>
       <c r="H40" s="21" t="n">
         <v>0.14</v>
@@ -33563,7 +33563,7 @@
         <v>0.22</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="O7" s="10" t="n">
         <v>1.01</v>
@@ -33733,7 +33733,7 @@
         <v>-0.5600000000000001</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>-0.23</v>
+        <v>-0.24</v>
       </c>
       <c r="Q9" s="10" t="n">
         <v>-0.08</v>
@@ -33791,34 +33791,34 @@
         <v>1.01</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>1.51</v>
+        <v>2.04</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>0.45</v>
+        <v>0.62</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>-0.35</v>
+        <v>0.18</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.39</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>-0.35</v>
+        <v>-0.26</v>
       </c>
       <c r="M10" s="9" t="n">
-        <v>-0.1</v>
+        <v>-0.08</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>-0.9</v>
+        <v>-0.37</v>
       </c>
       <c r="O10" s="9" t="n">
-        <v>-0.43</v>
+        <v>-0.26</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>-0.36</v>
+        <v>-0.27</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>-0.06</v>
+        <v>-0.03</v>
       </c>
       <c r="R10" s="9">
         <f>(H10-I10)-(F10-G10)</f>
@@ -33829,16 +33829,16 @@
         <v/>
       </c>
       <c r="T10" s="9" t="n">
-        <v>2.17</v>
+        <v>2.31</v>
       </c>
       <c r="U10" s="9" t="n">
         <v>1.94</v>
       </c>
       <c r="V10" s="9" t="n">
-        <v>0.22</v>
+        <v>0.37</v>
       </c>
       <c r="W10" s="9" t="n">
-        <v>12.52</v>
+        <v>12.67</v>
       </c>
       <c r="X10" s="9" t="n">
         <v>15.36</v>
@@ -34158,16 +34158,16 @@
         <v>2</v>
       </c>
       <c r="E38" s="19" t="n">
-        <v>-0.63</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="F38" s="19" t="n">
         <v>-0.9</v>
       </c>
       <c r="G38" s="19" t="n">
-        <v>-0.68</v>
+        <v>-0.54</v>
       </c>
       <c r="H38" s="19" t="n">
-        <v>-0.77</v>
+        <v>-0.33</v>
       </c>
     </row>
     <row r="39">
@@ -34214,16 +34214,16 @@
         <v>10</v>
       </c>
       <c r="E40" s="21" t="n">
-        <v>-0.49</v>
+        <v>-0.45</v>
       </c>
       <c r="F40" s="21" t="n">
         <v>-0.46</v>
       </c>
       <c r="G40" s="21" t="n">
-        <v>-0.38</v>
+        <v>-0.3</v>
       </c>
       <c r="H40" s="21" t="n">
-        <v>-0.33</v>
+        <v>-0.21</v>
       </c>
     </row>
   </sheetData>
@@ -34755,16 +34755,16 @@
         <v>-0.46</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>-0.45</v>
+        <v>-0.48</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>-0.18</v>
+        <v>-0.25</v>
       </c>
       <c r="P4" s="9" t="n">
         <v>0.01</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.42</v>
+        <v>-0.44</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -34843,10 +34843,10 @@
         <v>-0.19</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>-0.36</v>
+        <v>-0.38</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -34919,16 +34919,16 @@
         <v>-0.57</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-0.88</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>-0.66</v>
+        <v>-0.68</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.15</v>
+        <v>-0.17</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>-0.42</v>
+        <v>-0.44</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -35007,10 +35007,10 @@
         <v>0.12</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.15</v>
+        <v>-0.16</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>-0.33</v>
+        <v>-0.35</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -35083,16 +35083,16 @@
         <v>-0.65</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>1.41</v>
+        <v>1.4</v>
       </c>
       <c r="O8" s="9" t="n">
         <v>-0.44</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.37</v>
+        <v>-0.38</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -35171,10 +35171,10 @@
         <v>0.34</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>-0.02</v>
+        <v>-0.04</v>
       </c>
       <c r="Q9" s="10" t="n">
-        <v>-0.17</v>
+        <v>-0.18</v>
       </c>
       <c r="R9" s="10">
         <f>(H9-I9)-(F9-G9)</f>
@@ -35229,34 +35229,34 @@
         <v>1.84</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>1.1</v>
+        <v>1.13</v>
       </c>
       <c r="I10" s="9" t="n">
         <v>1.56</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="K10" s="9" t="n">
         <v>-0.28</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="M10" s="9" t="n">
         <v>-0.47</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="O10" s="9" t="n">
         <v>-0.74</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>-0.26</v>
+        <v>-0.27</v>
       </c>
       <c r="R10" s="9">
         <f>(H10-I10)-(F10-G10)</f>
@@ -35267,16 +35267,16 @@
         <v/>
       </c>
       <c r="T10" s="9" t="n">
-        <v>1.06</v>
+        <v>1.08</v>
       </c>
       <c r="U10" s="9" t="n">
         <v>0.82</v>
       </c>
       <c r="V10" s="9" t="n">
-        <v>0.23</v>
+        <v>0.26</v>
       </c>
       <c r="W10" s="9" t="n">
-        <v>13.69</v>
+        <v>13.72</v>
       </c>
       <c r="X10" s="9" t="n">
         <v>9.890000000000001</v>
@@ -35633,7 +35633,7 @@
         <v>-0.22</v>
       </c>
       <c r="H39" s="19" t="n">
-        <v>-0.17</v>
+        <v>-0.14</v>
       </c>
     </row>
     <row r="40">
@@ -35655,13 +35655,13 @@
         <v>0.65</v>
       </c>
       <c r="F40" s="21" t="n">
-        <v>0.42</v>
+        <v>0.43</v>
       </c>
       <c r="G40" s="21" t="n">
-        <v>-0.29</v>
+        <v>-0.28</v>
       </c>
       <c r="H40" s="21" t="n">
-        <v>-0.17</v>
+        <v>-0.14</v>
       </c>
     </row>
   </sheetData>
@@ -36521,16 +36521,16 @@
         <v>0.09</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>0.01</v>
+        <v>-0.01</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>-0.45</v>
+        <v>-0.52</v>
       </c>
       <c r="P8" s="9" t="n">
         <v>-0.12</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -36609,10 +36609,10 @@
         <v>-0.26</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="Q9" s="10" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="R9" s="10">
         <f>(H9-I9)-(F9-G9)</f>
@@ -36691,10 +36691,10 @@
         <v>0.85</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="R10" s="9">
         <f>(H10-I10)-(F10-G10)</f>
@@ -37470,13 +37470,13 @@
         <v>0.25</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="P2" s="9" t="n">
         <v>0.25</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -37713,13 +37713,13 @@
         <v>0.26</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>-0.48</v>
+        <v>-0.49</v>
       </c>
       <c r="O5" s="10" t="n">
         <v>0.77</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-0.05</v>
+        <v>-0.06</v>
       </c>
       <c r="Q5" s="10" t="n">
         <v>0.28</v>
@@ -37801,7 +37801,7 @@
         <v>0.47</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="Q6" s="9" t="n">
         <v>0.32</v>
@@ -37883,7 +37883,7 @@
         <v>0.26</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>0.31</v>
@@ -37962,7 +37962,7 @@
         <v>0.11</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>-0.76</v>
+        <v>-0.77</v>
       </c>
       <c r="P8" s="9" t="n">
         <v>0.1</v>
@@ -38987,7 +38987,7 @@
         <v>-0.2</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>-0.12</v>
+        <v>-0.13</v>
       </c>
       <c r="O3" s="10" t="n">
         <v>-0.89</v>
@@ -39157,7 +39157,7 @@
         <v>0.22</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
       <c r="Q5" s="10" t="n">
         <v>0.08</v>
@@ -39236,7 +39236,7 @@
         <v>-0.64</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="P6" s="9" t="n">
         <v>0.5600000000000001</v>
@@ -39406,7 +39406,7 @@
         <v>-0.04</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.01</v>
+        <v>-0.02</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -40264,13 +40264,13 @@
         <v>0.55</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="P2" s="9" t="n">
         <v>0.55</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -40343,13 +40343,13 @@
         <v>0.18</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>1.43</v>
+        <v>1.42</v>
       </c>
       <c r="O3" s="10" t="n">
         <v>-0.67</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="Q3" s="10" t="n">
         <v>0.04</v>
@@ -40428,13 +40428,13 @@
         <v>-0.27</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>-0.02</v>
+        <v>-0.03</v>
       </c>
       <c r="P4" s="9" t="n">
         <v>0.57</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -40595,10 +40595,10 @@
         <v>0.09</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -40759,7 +40759,7 @@
         <v>-0.12</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.45</v>
+        <v>0.44</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>-0.16</v>
@@ -43914,19 +43914,19 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Rotherham United</t>
+          <t>Newport County</t>
         </is>
       </c>
       <c r="C4" s="6">
-        <f>'Rotherham United'!$E$13</f>
+        <f>'Newport County'!$E$13</f>
         <v/>
       </c>
       <c r="D4" s="9">
-        <f>'Rotherham United'!$E$32</f>
+        <f>'Newport County'!$E$32</f>
         <v/>
       </c>
       <c r="E4" s="9">
-        <f>'Rotherham United'!$E$33</f>
+        <f>'Newport County'!$E$33</f>
         <v/>
       </c>
       <c r="F4" s="9">
@@ -43940,19 +43940,19 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Newport County</t>
+          <t>Rotherham United</t>
         </is>
       </c>
       <c r="C5" s="8">
-        <f>'Newport County'!$E$13</f>
+        <f>'Rotherham United'!$E$13</f>
         <v/>
       </c>
       <c r="D5" s="10">
-        <f>'Newport County'!$E$32</f>
+        <f>'Rotherham United'!$E$32</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>'Newport County'!$E$33</f>
+        <f>'Rotherham United'!$E$33</f>
         <v/>
       </c>
       <c r="F5" s="10">
@@ -44070,19 +44070,19 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Grimsby Town</t>
+          <t>Gillingham</t>
         </is>
       </c>
       <c r="C10" s="6">
-        <f>'Grimsby Town'!$E$13</f>
+        <f>'Gillingham'!$E$13</f>
         <v/>
       </c>
       <c r="D10" s="9">
-        <f>'Grimsby Town'!$E$32</f>
+        <f>'Gillingham'!$E$32</f>
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>'Grimsby Town'!$E$33</f>
+        <f>'Gillingham'!$E$33</f>
         <v/>
       </c>
       <c r="F10" s="9">
@@ -44096,19 +44096,19 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Gillingham</t>
+          <t>Grimsby Town</t>
         </is>
       </c>
       <c r="C11" s="8">
-        <f>'Gillingham'!$E$13</f>
+        <f>'Grimsby Town'!$E$13</f>
         <v/>
       </c>
       <c r="D11" s="10">
-        <f>'Gillingham'!$E$32</f>
+        <f>'Grimsby Town'!$E$32</f>
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>'Gillingham'!$E$33</f>
+        <f>'Grimsby Town'!$E$33</f>
         <v/>
       </c>
       <c r="F11" s="10">
@@ -50309,28 +50309,28 @@
         <v>1.01</v>
       </c>
       <c r="H97" s="10" t="n">
-        <v>1.51</v>
+        <v>2.04</v>
       </c>
       <c r="I97" s="10" t="n">
-        <v>0.45</v>
+        <v>0.62</v>
       </c>
       <c r="J97" s="10" t="n">
-        <v>-0.35</v>
+        <v>0.18</v>
       </c>
       <c r="K97" s="10" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.39</v>
       </c>
       <c r="L97" s="10" t="n">
-        <v>0.21</v>
+        <v>0.57</v>
       </c>
       <c r="M97" s="10" t="n">
-        <v>-0.91</v>
+        <v>-0.21</v>
       </c>
       <c r="N97" s="10" t="n">
-        <v>2.17</v>
+        <v>2.31</v>
       </c>
       <c r="O97" s="10" t="n">
-        <v>0.58</v>
+        <v>0.5</v>
       </c>
       <c r="P97" s="10" t="n">
         <v>1.94</v>
@@ -50368,28 +50368,28 @@
         <v>1.32</v>
       </c>
       <c r="H98" s="9" t="n">
-        <v>2.09</v>
+        <v>2.18</v>
       </c>
       <c r="I98" s="9" t="n">
         <v>0.47</v>
       </c>
       <c r="J98" s="9" t="n">
-        <v>0.76</v>
+        <v>0.85</v>
       </c>
       <c r="K98" s="9" t="n">
         <v>-0.85</v>
       </c>
       <c r="L98" s="9" t="n">
-        <v>1.61</v>
+        <v>1.7</v>
       </c>
       <c r="M98" s="9" t="n">
-        <v>-0.1</v>
+        <v>-0.01</v>
       </c>
       <c r="N98" s="9" t="n">
-        <v>2.44</v>
+        <v>2.47</v>
       </c>
       <c r="O98" s="9" t="n">
-        <v>0.39</v>
+        <v>0.36</v>
       </c>
       <c r="P98" s="9" t="n">
         <v>1.37</v>
@@ -50548,25 +50548,25 @@
         <v>1.56</v>
       </c>
       <c r="I101" s="10" t="n">
-        <v>1.1</v>
+        <v>1.13</v>
       </c>
       <c r="J101" s="10" t="n">
         <v>-0.28</v>
       </c>
       <c r="K101" s="10" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="L101" s="10" t="n">
-        <v>-0.4</v>
+        <v>-0.43</v>
       </c>
       <c r="M101" s="10" t="n">
-        <v>-0.17</v>
+        <v>-0.14</v>
       </c>
       <c r="N101" s="10" t="n">
-        <v>1.69</v>
+        <v>1.67</v>
       </c>
       <c r="O101" s="10" t="n">
-        <v>1.06</v>
+        <v>1.08</v>
       </c>
       <c r="P101" s="10" t="n">
         <v>1.95</v>
@@ -50663,28 +50663,28 @@
         <v>1.53</v>
       </c>
       <c r="H103" s="10" t="n">
-        <v>1.59</v>
+        <v>1.6</v>
       </c>
       <c r="I103" s="10" t="n">
-        <v>0.74</v>
+        <v>0.79</v>
       </c>
       <c r="J103" s="10" t="n">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="K103" s="10" t="n">
-        <v>-0.79</v>
+        <v>-0.74</v>
       </c>
       <c r="L103" s="10" t="n">
-        <v>1.14</v>
+        <v>1.1</v>
       </c>
       <c r="M103" s="10" t="n">
-        <v>-0.45</v>
+        <v>-0.39</v>
       </c>
       <c r="N103" s="10" t="n">
-        <v>1.98</v>
+        <v>1.95</v>
       </c>
       <c r="O103" s="10" t="n">
-        <v>0.77</v>
+        <v>0.8</v>
       </c>
       <c r="P103" s="10" t="n">
         <v>1.18</v>
@@ -50844,7 +50844,7 @@
         <v>0.65</v>
       </c>
       <c r="C4" s="10" t="n">
-        <v>0.42</v>
+        <v>0.43</v>
       </c>
       <c r="D4" s="10" t="n">
         <v>0.44</v>
@@ -50866,7 +50866,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.47</v>
+        <v>0.46</v>
       </c>
       <c r="C5" s="9" t="n">
         <v>0.57</v>
@@ -50878,7 +50878,7 @@
         <v>0.55</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>0.5</v>
+        <v>0.48</v>
       </c>
       <c r="G5" s="9" t="n">
         <v>0.57</v>
@@ -50941,13 +50941,13 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="C8" s="10" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>0.79</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E8" s="10" t="n">
         <v>1.06</v>
@@ -50966,7 +50966,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>0</v>
@@ -51106,7 +51106,7 @@
         <v>-0.71</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>-1.14</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="15">
@@ -51187,51 +51187,51 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Crewe Alexandra</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="B18" s="10" t="n">
         <v>-0.17</v>
       </c>
       <c r="C18" s="10" t="n">
-        <v>-0.28</v>
+        <v>-0.19</v>
       </c>
       <c r="D18" s="10" t="n">
-        <v>-0.62</v>
+        <v>0.4</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>-0.62</v>
+        <v>0.28</v>
       </c>
       <c r="F18" s="10" t="n">
-        <v>0.38</v>
+        <v>-0.63</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>0.24</v>
+        <v>-0.55</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Swindon Town</t>
+          <t>Crewe Alexandra</t>
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>-0.17</v>
+        <v>-0.18</v>
       </c>
       <c r="C19" s="9" t="n">
-        <v>-0.19</v>
+        <v>-0.28</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>0.4</v>
+        <v>-0.63</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>0.28</v>
+        <v>-0.62</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>-0.63</v>
+        <v>0.38</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>-0.55</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="20">
@@ -51316,13 +51316,13 @@
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>-0.49</v>
+        <v>-0.45</v>
       </c>
       <c r="C23" s="9" t="n">
         <v>-0.46</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>-0.63</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="E23" s="9" t="n">
         <v>-0.9</v>
@@ -51366,10 +51366,10 @@
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>-0.62</v>
+        <v>-0.66</v>
       </c>
       <c r="C25" s="9" t="n">
-        <v>-0.49</v>
+        <v>-0.57</v>
       </c>
       <c r="D25" s="9" t="n">
         <v>-0.55</v>
@@ -51378,10 +51378,10 @@
         <v>-0.54</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>-0.68</v>
+        <v>-0.75</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>-0.38</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="26">
@@ -51831,51 +51831,51 @@
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>Crewe Alexandra</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="B45" s="8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C45" s="8" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D45" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E45" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G45" s="8" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Swindon Town</t>
+          <t>Crewe Alexandra</t>
         </is>
       </c>
       <c r="B46" s="6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C46" s="6" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D46" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F46" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G46" s="6" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
@@ -52894,94 +52894,94 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Crewe Alexandra</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="B17" s="14">
-        <f>'Crewe Alexandra'!$E$24</f>
+        <f>'Swindon Town'!$E$24</f>
         <v/>
       </c>
       <c r="C17" s="9">
-        <f>'Crewe Alexandra'!$R$2</f>
+        <f>'Swindon Town'!$R$2</f>
         <v/>
       </c>
       <c r="D17" s="9">
-        <f>'Crewe Alexandra'!$R$3</f>
+        <f>'Swindon Town'!$R$3</f>
         <v/>
       </c>
       <c r="E17" s="9">
-        <f>'Crewe Alexandra'!$R$4</f>
+        <f>'Swindon Town'!$R$4</f>
         <v/>
       </c>
       <c r="F17" s="9">
-        <f>'Crewe Alexandra'!$R$5</f>
+        <f>'Swindon Town'!$R$5</f>
         <v/>
       </c>
       <c r="G17" s="9">
-        <f>'Crewe Alexandra'!$R$6</f>
+        <f>'Swindon Town'!$R$6</f>
         <v/>
       </c>
       <c r="H17" s="9">
-        <f>'Crewe Alexandra'!$R$7</f>
+        <f>'Swindon Town'!$R$7</f>
         <v/>
       </c>
       <c r="I17" s="9">
-        <f>'Crewe Alexandra'!$R$8</f>
+        <f>'Swindon Town'!$R$8</f>
         <v/>
       </c>
       <c r="J17" s="9">
-        <f>'Crewe Alexandra'!$R$9</f>
+        <f>'Swindon Town'!$R$9</f>
         <v/>
       </c>
       <c r="K17" s="9">
-        <f>'Crewe Alexandra'!$R$10</f>
+        <f>'Swindon Town'!$R$10</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Swindon Town</t>
+          <t>Crewe Alexandra</t>
         </is>
       </c>
       <c r="B18" s="14">
-        <f>'Swindon Town'!$E$24</f>
+        <f>'Crewe Alexandra'!$E$24</f>
         <v/>
       </c>
       <c r="C18" s="9">
-        <f>'Swindon Town'!$R$2</f>
+        <f>'Crewe Alexandra'!$R$2</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>'Swindon Town'!$R$3</f>
+        <f>'Crewe Alexandra'!$R$3</f>
         <v/>
       </c>
       <c r="E18" s="9">
-        <f>'Swindon Town'!$R$4</f>
+        <f>'Crewe Alexandra'!$R$4</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>'Swindon Town'!$R$5</f>
+        <f>'Crewe Alexandra'!$R$5</f>
         <v/>
       </c>
       <c r="G18" s="9">
-        <f>'Swindon Town'!$R$6</f>
+        <f>'Crewe Alexandra'!$R$6</f>
         <v/>
       </c>
       <c r="H18" s="9">
-        <f>'Swindon Town'!$R$7</f>
+        <f>'Crewe Alexandra'!$R$7</f>
         <v/>
       </c>
       <c r="I18" s="9">
-        <f>'Swindon Town'!$R$8</f>
+        <f>'Crewe Alexandra'!$R$8</f>
         <v/>
       </c>
       <c r="J18" s="9">
-        <f>'Swindon Town'!$R$9</f>
+        <f>'Crewe Alexandra'!$R$9</f>
         <v/>
       </c>
       <c r="K18" s="9">
-        <f>'Swindon Town'!$R$10</f>
+        <f>'Crewe Alexandra'!$R$10</f>
         <v/>
       </c>
     </row>

</xml_diff>